<commit_message>
cleaned some code and added mean pooling to SBERT / ROBERTA
</commit_message>
<xml_diff>
--- a/Datasets/cleaned_all_courses.xlsx
+++ b/Datasets/cleaned_all_courses.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B212"/>
+  <dimension ref="A1:B211"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2591,378 +2591,370 @@
     <row r="181">
       <c r="A181" t="inlineStr">
         <is>
-          <t>IDC_5007</t>
-        </is>
-      </c>
-      <c r="B181" t="inlineStr"/>
+          <t>IDC_6940</t>
+        </is>
+      </c>
+      <c r="B181" t="inlineStr">
+        <is>
+          <t>new course syllabus course title idc capstone course data science catalog description projects course using python sql r specialized analysis toolkits synthesize concepts data analytics visualization applied industry relevant projects credits prerequisites cap introduction data science type required course ms data science objectives goal course carry industry relevant project applied data science synthesizes concepts databases analytics visualization management data class meet biweekly learn analysis case histories monitor project progress class presentations evaluate project progress reports projects may involve individual team effort students assigned project mentor identify plan outline execute data science project students meet periodically project mentor discuss project progress results troubleshoot topics project selection planning designing database analytics visualization aspects project project presentations report writing textbook none</t>
+        </is>
+      </c>
     </row>
     <row r="182">
       <c r="A182" t="inlineStr">
         <is>
-          <t>IDC_6940</t>
+          <t>IDS_2916</t>
         </is>
       </c>
       <c r="B182" t="inlineStr">
         <is>
-          <t>new course syllabus course title idc capstone course data science catalog description projects course using python sql r specialized analysis toolkits synthesize concepts data analytics visualization applied industry relevant projects credits prerequisites cap introduction data science type required course ms data science objectives goal course carry industry relevant project applied data science synthesizes concepts databases analytics visualization management data class meet biweekly learn analysis case histories monitor project progress class presentations evaluate project progress reports projects may involve individual team effort students assigned project mentor identify plan outline execute data science project students meet periodically project mentor discuss project progress results troubleshoot topics project selection planning designing database analytics visualization aspects project project presentations report writing textbook none</t>
+          <t>knight foundation school computing information sciences course title vertically integrated projects date course number ids number credits catalog description students work large projects students different majors working real world projects university external mentors may taken twice sophomore status objective course understand teamwork real world scenarios develop complete solutions working inter disciplinary groups improve presentation writing skills learn domains course outcomes prepare research paper format appropriate particular field domain present visual summary research project using conventional display medium e g presentation slides poster demo etc give oral presentation findings scholarly work oral written communication written reports oral presentations required approx pages required approx time social ethical implications topics topic class time student performance measures citations plagiarism social impact throughout semester student presentations research papers problem analysis solution design experiences identify one problem student field would benefit research knight foundation school computing information sciences ids vertically integrated projects assessment plan course data course used assess program outcomes student instructor course outcome surveys administered conclusion offering evaluated described school assessment plan https abet cs fiu edu csassessment</t>
         </is>
       </c>
     </row>
     <row r="183">
       <c r="A183" t="inlineStr">
         <is>
-          <t>IDS_2916</t>
+          <t>IDS_3917</t>
         </is>
       </c>
       <c r="B183" t="inlineStr">
         <is>
-          <t>knight foundation school computing information sciences course title vertically integrated projects date course number ids number credits catalog description students work large projects students different majors working real world projects university external mentors may taken twice sophomore status objective course understand teamwork real world scenarios develop complete solutions working inter disciplinary groups improve presentation writing skills learn domains course outcomes prepare research paper format appropriate particular field domain present visual summary research project using conventional display medium e g presentation slides poster demo etc give oral presentation findings scholarly work oral written communication written reports oral presentations required approx pages required approx time social ethical implications topics topic class time student performance measures citations plagiarism social impact throughout semester student presentations research papers problem analysis solution design experiences identify one problem student field would benefit research knight foundation school computing information sciences ids vertically integrated projects assessment plan course data course used assess program outcomes student instructor course outcome surveys administered conclusion offering evaluated described school assessment plan https abet cs fiu edu csassessment</t>
+          <t>knight foundation school computing information sciences course title vertically integrated projects b date course number ids number credits catalog description students work large projects students different majors working real world projects university external mentors may taken twice junior status objective course understand teamwork real world scenarios develop complete solutions working inter disciplinary groups improve presentation writing skills learn domains course outcomes prepare research paper format appropriate particular field domain present visual summary research project using conventional display medium e g presentation slides poster demo etc give oral presentation findings scholarly work identify differing methodologies discovering new knowledge utilize libraries repositories find literature relevant specific research topic critique relevance importance previous work current research topic oral written communication written reports oral presentations required approx pages required approx time social ethical implications topics topic class time student performance measures citations plagiarism social impact throughout semester student presentations research papers privacy privacy protection throughout semester student presentations research papers knight foundation school computing information sciences ids vertically integrated projects b problem analysis solution design experiences identify one problem student field would benefit research write informal proposal research project based problem assessment plan course data course used assess program outcomes student instructor course outcome surveys administered conclusion offering evaluated described school assessment plan https abet cs fiu edu csassessment</t>
         </is>
       </c>
     </row>
     <row r="184">
       <c r="A184" t="inlineStr">
         <is>
-          <t>IDS_3917</t>
+          <t>IDS_4918</t>
         </is>
       </c>
       <c r="B184" t="inlineStr">
         <is>
-          <t>knight foundation school computing information sciences course title vertically integrated projects b date course number ids number credits catalog description students work large projects students different majors working real world projects university external mentors may taken twice junior status objective course understand teamwork real world scenarios develop complete solutions working inter disciplinary groups improve presentation writing skills learn domains course outcomes prepare research paper format appropriate particular field domain present visual summary research project using conventional display medium e g presentation slides poster demo etc give oral presentation findings scholarly work identify differing methodologies discovering new knowledge utilize libraries repositories find literature relevant specific research topic critique relevance importance previous work current research topic oral written communication written reports oral presentations required approx pages required approx time social ethical implications topics topic class time student performance measures citations plagiarism social impact throughout semester student presentations research papers privacy privacy protection throughout semester student presentations research papers knight foundation school computing information sciences ids vertically integrated projects b problem analysis solution design experiences identify one problem student field would benefit research write informal proposal research project based problem assessment plan course data course used assess program outcomes student instructor course outcome surveys administered conclusion offering evaluated described school assessment plan https abet cs fiu edu csassessment</t>
+          <t>knight foundation school computing information sciences course title vertically integrated projects c date course number ids number credits catalog description students work large projects students different majors working real world projects university external mentors may taken twice senior status objective course understand teamwork real world scenarios develop complete solutions working inter disciplinary groups improve presentation writing skills learn domains subject area coordinator masoud sadjadi email sadjadi fiu edu course outcomes prepare research paper format appropriate particular field domain present visual summary research project using conventional display medium e g presentation slides poster demo etc give oral presentation findings scholarly work identify differing methodologies discovering new knowledge utilize libraries repositories find literature relevant specific research topic critique relevance importance previous work current research topic discuss issues privacy confidentiality active research describe consequences strategies avoidance plagiarism demonstrate individual responsibility context collective effort articulate requirements successful collaborative effor demonstrate acquisition knowledge area outside one expertise oral written communication written reports oral presentations required approx pages required approx time social ethical implications topics topic class time student performance knight foundation school computing information sciences ids vertically integrated projects c measures citations plagiarism social impact throughout semester student presentations research papers privacy privacy protection throughout semester student presentations research papers intellectual property patents trademarks copyrights similar products licensing final product invited lecture given office technology management commercialization fiu student presentat ions research papers problem analysis solution design experiences identify one problem student field would benefit research write formal proposal research project based problem assessment plan course data course used assess program outcomes student instructor course outcome surveys administered conclusion offering evaluated described school assessment plan https abet cs fiu edu csassessment</t>
         </is>
       </c>
     </row>
     <row r="185">
       <c r="A185" t="inlineStr">
         <is>
-          <t>IDS_4918</t>
+          <t>MAD_2104</t>
         </is>
       </c>
       <c r="B185" t="inlineStr">
         <is>
-          <t>knight foundation school computing information sciences course title vertically integrated projects c date course number ids number credits catalog description students work large projects students different majors working real world projects university external mentors may taken twice senior status objective course understand teamwork real world scenarios develop complete solutions working inter disciplinary groups improve presentation writing skills learn domains subject area coordinator masoud sadjadi email sadjadi fiu edu course outcomes prepare research paper format appropriate particular field domain present visual summary research project using conventional display medium e g presentation slides poster demo etc give oral presentation findings scholarly work identify differing methodologies discovering new knowledge utilize libraries repositories find literature relevant specific research topic critique relevance importance previous work current research topic discuss issues privacy confidentiality active research describe consequences strategies avoidance plagiarism demonstrate individual responsibility context collective effort articulate requirements successful collaborative effor demonstrate acquisition knowledge area outside one expertise oral written communication written reports oral presentations required approx pages required approx time social ethical implications topics topic class time student performance knight foundation school computing information sciences ids vertically integrated projects c measures citations plagiarism social impact throughout semester student presentations research papers privacy privacy protection throughout semester student presentations research papers intellectual property patents trademarks copyrights similar products licensing final product invited lecture given office technology management commercialization fiu student presentat ions research papers problem analysis solution design experiences identify one problem student field would benefit research write formal proposal research project based problem assessment plan course data course used assess program outcomes student instructor course outcome surveys administered conclusion offering evaluated described school assessment plan https abet cs fiu edu csassessment</t>
+          <t>knight foundation school comput ing information science course title discrete mathematic date course number mad number credits subject area foundations subject area coordinator hadi amini email amini cs fiu edu catalog description sets functions relations permutations combinations propositional logic matrix algebra graphs trees boolean algebra switching circuits typical textbook kenneth rosen discrete mathematics applications th edition mcgraw hill references prerequisite course none corequisite courses cop type required prerequisites topics course outcome master definitions theorems involving sets relations functions familiar propositional logic familiar mathematical reasoning including mathematical induction recursion exposed combinatoric familiar graph theory exposed boolean algebras knig ht foundation school com puting information sciences mad discrete mathematics outline topic number lecture hours outcome sets relations functions operations sets equivalence relations cardinality logic mathematical reasoning propositional logic mathematical induction recursion combinatorics combinatorial identities binomial theorem directed undirected graphs isomorphism graphs paths adjacency matrices euler paths four color problem planar graphs trees tree traversal boolean algebras disjunct ive n ormal form minimization boolean f unctions karnaugh maps course outcomes emphasized laboratory projects assignments outcome number weeks oral written communicati significant c overa ge knig ht foundation school com puting information sciences mad discrete mathematics social e thical implications computing topics significant coverage approximate number credit hours devoted fundamental cs topics topic core hours advanced hours algorithms software design computer organization arch itecture data structures concepts programming languages theoretical contents topic class time discrete structures hours problem analysis experiences significant coverage solution design experiences signi ficant coverage appr oxima te number credit hours devoted fundamental cs topics topic core hours advanced hours algorithms software design computer organization architectur e data structures concepts programming languages knig ht foundation school com puting information sciences mad discrete mathematics theoretical cont ents topic class time discrete structures hours problem analysis experiences significant coverage solution design experiences significant coverage coverage knowledge units within computer science body knowledge knowledge unit topi c lecture hours ds functions relations sets ds basic logic ds proof techniques ds basics counting ds graphs trees assessment plan course data course used assess progr ou tcomes student instructor course outcome surveys administered conclusion offering evaluated described school assessment plan https abet cs fiu edu csa ssess ment see https www acm org binaries content assets education cs web final pdf description computer science knowledge units</t>
         </is>
       </c>
     </row>
     <row r="186">
       <c r="A186" t="inlineStr">
         <is>
-          <t>MAD_2104</t>
+          <t>MAD_3301</t>
         </is>
       </c>
       <c r="B186" t="inlineStr">
         <is>
-          <t>knight foundation school comput ing information science course title discrete mathematic date course number mad number credits subject area foundations subject area coordinator hadi amini email amini cs fiu edu catalog description sets functions relations permutations combinations propositional logic matrix algebra graphs trees boolean algebra switching circuits typical textbook kenneth rosen discrete mathematics applications th edition mcgraw hill references prerequisite course none corequisite courses cop type required prerequisites topics course outcome master definitions theorems involving sets relations functions familiar propositional logic familiar mathematical reasoning including mathematical induction recursion exposed combinatoric familiar graph theory exposed boolean algebras knig ht foundation school com puting information sciences mad discrete mathematics outline topic number lecture hours outcome sets relations functions operations sets equivalence relations cardinality logic mathematical reasoning propositional logic mathematical induction recursion combinatorics combinatorial identities binomial theorem directed undirected graphs isomorphism graphs paths adjacency matrices euler paths four color problem planar graphs trees tree traversal boolean algebras disjunct ive n ormal form minimization boolean f unctions karnaugh maps course outcomes emphasized laboratory projects assignments outcome number weeks oral written communicati significant c overa ge knig ht foundation school com puting information sciences mad discrete mathematics social e thical implications computing topics significant coverage approximate number credit hours devoted fundamental cs topics topic core hours advanced hours algorithms software design computer organization arch itecture data structures concepts programming languages theoretical contents topic class time discrete structures hours problem analysis experiences significant coverage solution design experiences signi ficant coverage appr oxima te number credit hours devoted fundamental cs topics topic core hours advanced hours algorithms software design computer organization architectur e data structures concepts programming languages knig ht foundation school com puting information sciences mad discrete mathematics theoretical cont ents topic class time discrete structures hours problem analysis experiences significant coverage solution design experiences significant coverage coverage knowledge units within computer science body knowledge knowledge unit topi c lecture hours ds functions relations sets ds basic logic ds proof techniques ds basics counting ds graphs trees assessment plan course data course used assess progr ou tcomes student instructor course outcome surveys administered conclusion offering evaluated described school assessment plan https abet cs fiu edu csa ssess ment see https www acm org binaries content assets education cs web final pdf description computer science knowledge units</t>
+          <t>knight foundati school comput ing information science course title graph theory date course number mad number credits subject area foundations subject area coordinator hadi amini email amini cs fiu edu catalog des cription introduction study graphs topics include following paths circuits connectedness trees shortest paths networks planar graphs coloring graphs directed graphs applications graphs comput er science discussed textbook references prerequisite course cop cgs either mas mad corequisite courses none type elective cs foundations group prerequisites topics course outcome master p aths connectedness directed u ndirected graphs master graphs trees master shortest path algorithms weighted unweighted graphs familiar planar colored graphs familiar applications graphs computer scien ce knig ht foundation school computing information sciences mad graph theory relationship course outcomes program outcomes bs cs program outcome course outcomes demonstrate proficiency foundation areas computer science including mathematics discrete struct ures logic theory algorithms b demonstrate proficiency various areas computer science including data structures algorithms concepts programming languages computer systems c demonstrate prof iciency problem solving application software engineering techniques demonstrate mastery least one modern programming language proficiency least one e demonstrate understanding social ethical concerns practicing computer sci entist f demonstrate ability work cooperatively teams g demonstrate effective communication skills assessment plan course data course used assess program outcomes student instructor course utcome surveys administered conclusion offering evaluated described school assessment plan https abet cs fiu edu csassessmen outline topic number lectu hours outcome knig ht foundation school computing information sciences mad graph theory course outcomes emp hasized laboratory projects assignments outcome number weeks oral written communication significant coverage written reports oral presentations number required approx number pages number required approx time social e thical mplications computing topics significant coverage topic class time student performance measures approximate number c redit hours devoted fundamenta l cs topics fundamental cs area core hours advanced hours algorithms software design computer organization architecture data structures concepts programming languages theoretical contents topic class time graph theory hours knig ht foundation school computing information sciences mad graph theory problem analy sis experiences solution design experiences coverage knowledge units within computer science body knowledge knowledge unit topic lecture hours see https www acm org binaries content assets education cs web final pdf description computer science knowledge units</t>
         </is>
       </c>
     </row>
     <row r="187">
       <c r="A187" t="inlineStr">
         <is>
-          <t>MAD_3301</t>
+          <t>MAD_3305</t>
         </is>
       </c>
       <c r="B187" t="inlineStr">
         <is>
-          <t>knight foundati school comput ing information science course title graph theory date course number mad number credits subject area foundations subject area coordinator hadi amini email amini cs fiu edu catalog des cription introduction study graphs topics include following paths circuits connectedness trees shortest paths networks planar graphs coloring graphs directed graphs applications graphs comput er science discussed textbook references prerequisite course cop cgs either mas mad corequisite courses none type elective cs foundations group prerequisites topics course outcome master p aths connectedness directed u ndirected graphs master graphs trees master shortest path algorithms weighted unweighted graphs familiar planar colored graphs familiar applications graphs computer scien ce knig ht foundation school computing information sciences mad graph theory relationship course outcomes program outcomes bs cs program outcome course outcomes demonstrate proficiency foundation areas computer science including mathematics discrete struct ures logic theory algorithms b demonstrate proficiency various areas computer science including data structures algorithms concepts programming languages computer systems c demonstrate prof iciency problem solving application software engineering techniques demonstrate mastery least one modern programming language proficiency least one e demonstrate understanding social ethical concerns practicing computer sci entist f demonstrate ability work cooperatively teams g demonstrate effective communication skills assessment plan course data course used assess program outcomes student instructor course utcome surveys administered conclusion offering evaluated described school assessment plan https abet cs fiu edu csassessmen outline topic number lectu hours outcome knig ht foundation school computing information sciences mad graph theory course outcomes emp hasized laboratory projects assignments outcome number weeks oral written communication significant coverage written reports oral presentations number required approx number pages number required approx time social e thical mplications computing topics significant coverage topic class time student performance measures approximate number c redit hours devoted fundamenta l cs topics fundamental cs area core hours advanced hours algorithms software design computer organization architecture data structures concepts programming languages theoretical contents topic class time graph theory hours knig ht foundation school computing information sciences mad graph theory problem analy sis experiences solution design experiences coverage knowledge units within computer science body knowledge knowledge unit topic lecture hours see https www acm org binaries content assets education cs web final pdf description computer science knowledge units</t>
+          <t>knight foundation school comput ing information science course title graph theory date course number mad mad number credits subject area foundations subject area coordinator hadi amini email amini cs fiu edu catalog description introduction study graphs topics include following paths circuits connectedness trees shortest paths networks planar graphs coloring graphs directed graphs applications graphs computer science discussed textbook references prerequisite course cop cgs either mas mad corequisite courses none type elective cs foundations group prerequisites topics course outcome master paths connectedness directed undirected graphs master graphs trees master shortest path algorithms weighted unweighted graphs familiar planar colored graphs familiar applications graphs computer science knight foundation school computing information sciences mad mad graph heory relationship course outcomes program outcomes bs cs program outcome course outcomes demonstrate proficiency foundation areas computer science including mathematics discrete structures logic theory algorithms b demonstrate proficiency various areas computer science including data structures algorithms concepts programming languages computer systems c demonstrate proficien cy problem solving application software engineering techniques demonstrate mastery least one modern programming language proficiency least one e demonstrate understanding social ethical concerns th e practicing computer scientist f demonstrate ability work cooperatively teams g demonstrate effective communication skills assessment plan course data course used assess program outcomes studen instructor course outcome surveys administered conclusion offering evaluated described school assessment plan https abet cs fiu edu csassessment outl ine topic number lecture hours outcome knight foundation school computing information sciences mad mad graph heory course outcomes emphasized laboratory projects assignments outcome number weeks oral written communication significant coverage written reports oral presentations number required appro x number pages number required approx time social e thical mplications computing topics significant coverage topic class time student performance measures approximate number c redit hours devoted fundamental c topics fundamental cs area core hours advanced hours algorithms software design computer organization architecture data structures concepts programming languages theoretical contents topic class time graph theory hours knight foundation school computing information sciences mad mad graph heory problem analysis experiences solution design experiences coverage knowledge units within computer science body knowledge knowledge unit topic lecture hours see https www acm org binaries content assets education cs web final pdf description computer science knowledge units</t>
         </is>
       </c>
     </row>
     <row r="188">
       <c r="A188" t="inlineStr">
         <is>
-          <t>MAD_3305</t>
+          <t>MAD_3401</t>
         </is>
       </c>
       <c r="B188" t="inlineStr">
         <is>
-          <t>knight foundation school comput ing information science course title graph theory date course number mad mad number credits subject area foundations subject area coordinator hadi amini email amini cs fiu edu catalog description introduction study graphs topics include following paths circuits connectedness trees shortest paths networks planar graphs coloring graphs directed graphs applications graphs computer science discussed textbook references prerequisite course cop cgs either mas mad corequisite courses none type elective cs foundations group prerequisites topics course outcome master paths connectedness directed undirected graphs master graphs trees master shortest path algorithms weighted unweighted graphs familiar planar colored graphs familiar applications graphs computer science knight foundation school computing information sciences mad mad graph heory relationship course outcomes program outcomes bs cs program outcome course outcomes demonstrate proficiency foundation areas computer science including mathematics discrete structures logic theory algorithms b demonstrate proficiency various areas computer science including data structures algorithms concepts programming languages computer systems c demonstrate proficien cy problem solving application software engineering techniques demonstrate mastery least one modern programming language proficiency least one e demonstrate understanding social ethical concerns th e practicing computer scientist f demonstrate ability work cooperatively teams g demonstrate effective communication skills assessment plan course data course used assess program outcomes studen instructor course outcome surveys administered conclusion offering evaluated described school assessment plan https abet cs fiu edu csassessment outl ine topic number lecture hours outcome knight foundation school computing information sciences mad mad graph heory course outcomes emphasized laboratory projects assignments outcome number weeks oral written communication significant coverage written reports oral presentations number required appro x number pages number required approx time social e thical mplications computing topics significant coverage topic class time student performance measures approximate number c redit hours devoted fundamental c topics fundamental cs area core hours advanced hours algorithms software design computer organization architecture data structures concepts programming languages theoretical contents topic class time graph theory hours knight foundation school computing information sciences mad mad graph heory problem analysis experiences solution design experiences coverage knowledge units within computer science body knowledge knowledge unit topic lecture hours see https www acm org binaries content assets education cs web final pdf description computer science knowledge units</t>
+          <t>knight foundation school comput ing information science course title numerical analysis date course number mad number credits subject area foundations subject area coordinator hadi amini email amini cs fiu edu catal og description basic ideas techniques numerical analysis topics include finite differences interpolation solution equations numerical integration differentiation applications introduction applied linear algebra thi cou rse ke extensive laboratory use computer facility textbook references prerequisite course cop cgs mac corequisite courses none type elective cs foundations group prerequisites topics course outcome master algorithms find ro ots equations interpola tion master numerical differentiation master numerical integration familiar finite differences familiar numerical solutions differential equations familiar numerical error analysis master writing progr solutions using techniques knig ht foundation school computing informatio n sciences mad numeri cal nalysis relationship course outcomes program outcomes bs cs program outcome course outcomes demonstrate profic iency foundation areas computer science including mathematics discr ete structures logic theory algorithms b demonstrate proficiency various areas computer science including data structures algorithms concepts programming languages computer systems c demonstrate proficien cy problem solving application software engineering techniques demonstrate mastery least one modern programming language proficiency least one e demonstrate understanding social ethical concerns th e practicing computer scientist f demonstrate ability work cooperatively teams g demonstrate effective communication skills assessment plan course data course used assess pr ogram outcomes studen instructor course outcome surveys administered conclusion offering evaluated described school assessment plan https abet cs fiu edu c sassessment outl ine topic number lecture hours outcome knig ht foundation school computing informatio n sciences mad numeri cal nalysis course outcomes emphasized laboratory projects assignments outcome number weeks oral written communication significant coverage written repor ts oral presentati ons number required approx number pages number required approx time social e thical implications computing topics significant coverage topic class time student performance measures approximate number c redit hour dev oted fundamental cs topics fundamental cs area core hours advanced hours algorithms software design computer organization architecture data structures concepts programming languages theoretical contents topic class time numerical analysi hours knig ht foundation school computing informatio n sciences mad numeri cal nalysis problem analysis experiences solution design experiences coverage knowledge units within computer science body knowledge knowledge unit topic lecture hours see https www acm org binaries content assets education cs web final pdf description computer science knowledge units</t>
         </is>
       </c>
     </row>
     <row r="189">
       <c r="A189" t="inlineStr">
         <is>
-          <t>MAD_3401</t>
+          <t>MAD_3512</t>
         </is>
       </c>
       <c r="B189" t="inlineStr">
         <is>
-          <t>knight foundation school comput ing information science course title numerical analysis date course number mad number credits subject area foundations subject area coordinator hadi amini email amini cs fiu edu catal og description basic ideas techniques numerical analysis topics include finite differences interpolation solution equations numerical integration differentiation applications introduction applied linear algebra thi cou rse ke extensive laboratory use computer facility textbook references prerequisite course cop cgs mac corequisite courses none type elective cs foundations group prerequisites topics course outcome master algorithms find ro ots equations interpola tion master numerical differentiation master numerical integration familiar finite differences familiar numerical solutions differential equations familiar numerical error analysis master writing progr solutions using techniques knig ht foundation school computing informatio n sciences mad numeri cal nalysis relationship course outcomes program outcomes bs cs program outcome course outcomes demonstrate profic iency foundation areas computer science including mathematics discr ete structures logic theory algorithms b demonstrate proficiency various areas computer science including data structures algorithms concepts programming languages computer systems c demonstrate proficien cy problem solving application software engineering techniques demonstrate mastery least one modern programming language proficiency least one e demonstrate understanding social ethical concerns th e practicing computer scientist f demonstrate ability work cooperatively teams g demonstrate effective communication skills assessment plan course data course used assess pr ogram outcomes studen instructor course outcome surveys administered conclusion offering evaluated described school assessment plan https abet cs fiu edu c sassessment outl ine topic number lecture hours outcome knig ht foundation school computing informatio n sciences mad numeri cal nalysis course outcomes emphasized laboratory projects assignments outcome number weeks oral written communication significant coverage written repor ts oral presentati ons number required approx number pages number required approx time social e thical implications computing topics significant coverage topic class time student performance measures approximate number c redit hour dev oted fundamental cs topics fundamental cs area core hours advanced hours algorithms software design computer organization architecture data structures concepts programming languages theoretical contents topic class time numerical analysi hours knig ht foundation school computing informatio n sciences mad numeri cal nalysis problem analysis experiences solution design experiences coverage knowledge units within computer science body knowledge knowledge unit topic lecture hours see https www acm org binaries content assets education cs web final pdf description computer science knowledge units</t>
+          <t>knight foun dation school comput ing forma tion science course title theory algorithms date course number mad number credits subject area foundations subject area coordinator hadi amini email amini cs fiu ed u catalog description strings formal languages finite state machines turing machines primitive recursive recursive functions recursive unsolvability typical textbook peter linz introduction formal languages automata third edition jones bartlett references prerequisite course cop corequisite courses none type elective cs foundations group prerequisites topics familiar ity w ith definitions theorems involving sets relations functions familiarity mathematical induction recurs ion familiarity formal proofs course outcome familiar formal languages master finite state machines master tur ing achines familiar w ith primitive recursive recursive functions exposed recursive unsolvability knig ht foundation school computing information sciences mad theo ry algorithms outline topic number lecture hours outcome regular languages regular expressions regular grammars deterministic finite automata nondet ermin istic finite automata minimizing dfas closure decidability properties pumping lemma regular languages context free languages context free grammars parsing ambiguity recursive recursively enumerable languages turing mach ines church turing thesis universal turing machine undecid able problems models computation recursive functions primitive recursive functions course outcomes emphasized laboratory projects assignments outcome numb er weeks oral written c ommunication significant coverage social e thical implications computing topics significant coverage knig ht foundation school computing information sciences mad theo ry algorithms approximate number credit hours devoted fundamental cs topics topi c core hours advanced hours algorithms software design computer organization architecture data structures concepts programming languages theoretical contents topic class time formal languages automata hours problem analysis experie nces significant coverage solution design experiences significant coverage coverage knowledge units within computer science body knowledge knowledge unit topic lecture hours al basic computability al automata theor assessment plan course data course used assess program outcomes student instructor course outcome surveys administered conclusion offering evaluated des cribed school assessment plan https abet cs fiu edu csassessment see https www acm org binarie content assets education cs web final pdf description computer science knowledge units</t>
         </is>
       </c>
     </row>
     <row r="190">
       <c r="A190" t="inlineStr">
         <is>
-          <t>MAD_3512</t>
+          <t>MAD_4203</t>
         </is>
       </c>
       <c r="B190" t="inlineStr">
         <is>
-          <t>knight foun dation school comput ing forma tion science course title theory algorithms date course number mad number credits subject area foundations subject area coordinator hadi amini email amini cs fiu ed u catalog description strings formal languages finite state machines turing machines primitive recursive recursive functions recursive unsolvability typical textbook peter linz introduction formal languages automata third edition jones bartlett references prerequisite course cop corequisite courses none type elective cs foundations group prerequisites topics familiar ity w ith definitions theorems involving sets relations functions familiarity mathematical induction recurs ion familiarity formal proofs course outcome familiar formal languages master finite state machines master tur ing achines familiar w ith primitive recursive recursive functions exposed recursive unsolvability knig ht foundation school computing information sciences mad theo ry algorithms outline topic number lecture hours outcome regular languages regular expressions regular grammars deterministic finite automata nondet ermin istic finite automata minimizing dfas closure decidability properties pumping lemma regular languages context free languages context free grammars parsing ambiguity recursive recursively enumerable languages turing mach ines church turing thesis universal turing machine undecid able problems models computation recursive functions primitive recursive functions course outcomes emphasized laboratory projects assignments outcome numb er weeks oral written c ommunication significant coverage social e thical implications computing topics significant coverage knig ht foundation school computing information sciences mad theo ry algorithms approximate number credit hours devoted fundamental cs topics topi c core hours advanced hours algorithms software design computer organization architecture data structures concepts programming languages theoretical contents topic class time formal languages automata hours problem analysis experie nces significant coverage solution design experiences significant coverage coverage knowledge units within computer science body knowledge knowledge unit topic lecture hours al basic computability al automata theor assessment plan course data course used assess program outcomes student instructor course outcome surveys administered conclusion offering evaluated des cribed school assessment plan https abet cs fiu edu csassessment see https www acm org binarie content assets education cs web final pdf description computer science knowledge units</t>
+          <t>knight foundation school comput ing information science course title introduction combinatorics date course number mad number credits subject area foundations subject area coordinator hadi amini email amini cs fiu edu catalog description survey basic techniques combinatorial mathematics topics include pigeonhole principle binomial coefficients inclusion exclusion recurrence relations generating functions textbook references prerequisite course mac mac mad corequisite courses none type elective cs foundations group prerequisites topics course outcome master basic techniques combinatorics pigeonhole principle binomial coefficients inclusi exclusion principle master basic techniques solving recurrence relations familiar generating functions applications knig ht foundation school com puting information sciences mad introduction combinatorics relation ship course outcomes program outcomes bs cs program outcome course outco mes demonstrate pr oficiency foundation areas computer science including mathematics discrete structures logic theory algorithms b demonstrate proficiency various areas computer science including data struct ures algorithms concepts programming languages computer systems c demonstrate proficiency problem solving application software engineering echniques demonstrate mastery least one modern programming language pr oficiency least one ther e demonstrate understanding social ethical concerns practicing computer scientist f demonstrate ability work cooperatively teams g demonstrate effective communication skills assessment plan course data course used assess program outcomes student instructor course outcome surveys administered conclusion offering evaluated described school assessment plan https abet cs fiu edu csassessment outline topic number lecture hours outcome knig ht foundation school com puting information sciences mad introduction combinatorics course outcomes emphasized laboratory projects assignments outcome number weeks oral writ ten communication significant coverage written reports oral presentations number required approx number pages number required approx time social e thical implications computing topics significant coverage topic class time student performa nce measures approximate number c redit hours devoted fundamental cs topics fundamental cs area core hours advanced hours algorithms software design computer organization architecture data struc tures concepts prog ramming languages theoretical contents topic class time combinatorics hours knig ht foundation school com puting information sciences mad introduction combinatorics problem analysis experiences solution design experiences coverage knowledge units within computer science body knowle dge knowledge unit topic lecture hours see https www acm org binaries content assets education cs web final pdf description computer science knowledge units</t>
         </is>
       </c>
     </row>
     <row r="191">
       <c r="A191" t="inlineStr">
         <is>
-          <t>MAD_4203</t>
+          <t>MHF_4302</t>
         </is>
       </c>
       <c r="B191" t="inlineStr">
         <is>
-          <t>knight foundation school comput ing information science course title introduction combinatorics date course number mad number credits subject area foundations subject area coordinator hadi amini email amini cs fiu edu catalog description survey basic techniques combinatorial mathematics topics include pigeonhole principle binomial coefficients inclusion exclusion recurrence relations generating functions textbook references prerequisite course mac mac mad corequisite courses none type elective cs foundations group prerequisites topics course outcome master basic techniques combinatorics pigeonhole principle binomial coefficients inclusi exclusion principle master basic techniques solving recurrence relations familiar generating functions applications knig ht foundation school com puting information sciences mad introduction combinatorics relation ship course outcomes program outcomes bs cs program outcome course outco mes demonstrate pr oficiency foundation areas computer science including mathematics discrete structures logic theory algorithms b demonstrate proficiency various areas computer science including data struct ures algorithms concepts programming languages computer systems c demonstrate proficiency problem solving application software engineering echniques demonstrate mastery least one modern programming language pr oficiency least one ther e demonstrate understanding social ethical concerns practicing computer scientist f demonstrate ability work cooperatively teams g demonstrate effective communication skills assessment plan course data course used assess program outcomes student instructor course outcome surveys administered conclusion offering evaluated described school assessment plan https abet cs fiu edu csassessment outline topic number lecture hours outcome knig ht foundation school com puting information sciences mad introduction combinatorics course outcomes emphasized laboratory projects assignments outcome number weeks oral writ ten communication significant coverage written reports oral presentations number required approx number pages number required approx time social e thical implications computing topics significant coverage topic class time student performa nce measures approximate number c redit hours devoted fundamental cs topics fundamental cs area core hours advanced hours algorithms software design computer organization architecture data struc tures concepts prog ramming languages theoretical contents topic class time combinatorics hours knig ht foundation school com puting information sciences mad introduction combinatorics problem analysis experiences solution design experiences coverage knowledge units within computer science body knowle dge knowledge unit topic lecture hours see https www acm org binaries content assets education cs web final pdf description computer science knowledge units</t>
+          <t>knight f oundation school comput ing information science course title mathematical logic date course number mhf number credits subject area foundations subject area coordinator hadi amini email amini cs fiu edu catal og description study formal logical systems applications foundations mathematics topics selected following definition mathematical proofs set theory analysis formalized predicate calculus theorem g del church recursive function theory idealized computers textbook references prerequisite course maa mad corequisite courses none type elective cs foundations group prerequisites topics course outcome master formal proofs propositional predicate logic master logical concepts sound ness completeness familiar applications logic foundations mathematics set theory analysis familiar limitative results g del church knig ht foundation school computing information sciences mhf mathemati cal logic relationship course outcomes program outcom es bs cs program come course outcomes demonstrate proficiency foundation areas computer science including mathematics discrete structures logic theory algorithms b demonstrate proficiency various area computer science inclu ding data structures algorithms concepts programming languages compute r systems c demonstrate proficiency problem solving application software engineering techniques demonstrate mastery le ast one modern programming language proficiency least one e demonstrate understanding f social ethical concerns practicing computer scientist f demonstrate ability work cooperatively teams g demon strate effective communicat ion skills assessment plan course data course used assess program outcomes student instructor course outcome surveys administered conclusion offering evaluat ed described scho ol assessment plan https abet cs fiu edu csassessment knig ht foundation school computing information sciences mhf mathemati cal logic outline topic number lecture hours outcome course outcomes emphasized laboratory projects assign ments outcome number eks oral written communication significant coverage written reports oral presentations number required approx number pages num ber required approx time social e thical implications compu ting topics significant coverage topic class time student performance measures appr oximate number c redit hours devoted fundamental cs topics fundamental cs area core hours advanced hours algorithms software design computer orga nizat ion architecture data structures concepts programming languages theoretical contents knig ht foundation school computing information sciences mhf mathemati cal logic topic class time mathematical logic hours problem analysis experiences solution design experiences coverage knowled ge un wi thin computer sc ience body knowledge knowledge unit topic lecture hours see https www acm org binaries content assets education cs web final pdf description com puter scien ce knowledge uni ts</t>
         </is>
       </c>
     </row>
     <row r="192">
       <c r="A192" t="inlineStr">
         <is>
-          <t>MHF_4302</t>
+          <t>STA_2122</t>
         </is>
       </c>
       <c r="B192" t="inlineStr">
         <is>
-          <t>knight f oundation school comput ing information science course title mathematical logic date course number mhf number credits subject area foundations subject area coordinator hadi amini email amini cs fiu edu catal og description study formal logical systems applications foundations mathematics topics selected following definition mathematical proofs set theory analysis formalized predicate calculus theorem g del church recursive function theory idealized computers textbook references prerequisite course maa mad corequisite courses none type elective cs foundations group prerequisites topics course outcome master formal proofs propositional predicate logic master logical concepts sound ness completeness familiar applications logic foundations mathematics set theory analysis familiar limitative results g del church knig ht foundation school computing information sciences mhf mathemati cal logic relationship course outcomes program outcom es bs cs program come course outcomes demonstrate proficiency foundation areas computer science including mathematics discrete structures logic theory algorithms b demonstrate proficiency various area computer science inclu ding data structures algorithms concepts programming languages compute r systems c demonstrate proficiency problem solving application software engineering techniques demonstrate mastery le ast one modern programming language proficiency least one e demonstrate understanding f social ethical concerns practicing computer scientist f demonstrate ability work cooperatively teams g demon strate effective communicat ion skills assessment plan course data course used assess program outcomes student instructor course outcome surveys administered conclusion offering evaluat ed described scho ol assessment plan https abet cs fiu edu csassessment knig ht foundation school computing information sciences mhf mathemati cal logic outline topic number lecture hours outcome course outcomes emphasized laboratory projects assign ments outcome number eks oral written communication significant coverage written reports oral presentations number required approx number pages num ber required approx time social e thical implications compu ting topics significant coverage topic class time student performance measures appr oximate number c redit hours devoted fundamental cs topics fundamental cs area core hours advanced hours algorithms software design computer orga nizat ion architecture data structures concepts programming languages theoretical contents knig ht foundation school computing information sciences mhf mathemati cal logic topic class time mathematical logic hours problem analysis experiences solution design experiences coverage knowled ge un wi thin computer sc ience body knowledge knowledge unit topic lecture hours see https www acm org binaries content assets education cs web final pdf description com puter scien ce knowledge uni ts</t>
+          <t>sta tr instructor leonid bekker home page http faculty fiu edu bekkerl phone email bekkerl fiu edu office ai office hours mw mw tr course objectives upon successful completion course students able apply working knowledge basic concepts used statistics interpret statistics used journal articles field demonstrate familiarity interpreting output statistical software package build upon foundation work statistics textbook using interactive statistics nd edition michael sullivan iii george woodbury nd mylab mylab guided notebook guided notebook alone students required purchase companion guided notebook interactive statistics exam coverage exam statistical thinking concepts descriptive statistics basic probability chapters exam discrete random variables binomial distribution continuous random variables normal distribution sampling distributions central limit theorem chapters exam confidence intervals hypothesis testing chapters final exam cumulative calculator students may use standard basic scientific calculators drop date march student whose name appears class list date receive letter grade course make policy assignments due indicated unforeseen emergency arises prev ents taking exam documentation must provided e summons jury duty letter physicians letterhead stating explicitly student could hand ass ignment take exam etc course communication contact via canvas mail directly bekkerl fiu edu online assignments include interactive assignments online homework chapter q uizzes chapter exams assigned homework quizzes tests except final exam must completed mystatlab integrated canvas attention proceed next chapter hw previous one accomplished least score prerequisite set every quiz test corresponding chapter hw accomplished least score exams scheduled three online chapter exams cumulative final exam class grading policy course requirements weights interactive assignments online homework quizzes exam exam exam final exam average hw score exceed extra points added final course score following scale basis assigning final grades grade range grade range grade range b c b b c f classroom policies classroom attendance necessary part course students unexcused absences rewarded extra points added final exam score lecture allowed use computers ipads cell phones etc course calendar assignment name date due sections covered introduction ia terminology types data qualitative quantitative types observational studies level measurement hw ia bar graph pie chart shape distribution dot plot histogram quiz ch quiz ch hw ia measures central tendency measures dispersion hw ia percentiles box plots quiz ch hw ia probability sample space union intersection complementary events hw ia additive multiplicative rules conditional probability independent dependent events quiz ch test online hw ia hw discrete random variable binomial random variable ia hw ia poisson random variable quiz ch hw ia continuous random variable normal distribution hw ia quiz ch hw ia sampling distribution mean proportion hw ia confidence interval academic integrity honesty form cheating academic dishonesty strictly forbidden class student found responsible academic misconduct subject academic misconduct procedures sanctions outlined student handbook signature enrolling class agreeing governed po licies syllabus also stating aware syllabus accompanying course calendar schedule subject change needed accommodate unforeseen issues arise term changes announced class posted canvas important read posted announcements daily quiz ch test online ia hw confidence interval proportion population mean hw ia test hypothesis terminology quiz ch hw ia b hw b ia test hypothesis proportion p hw test hypothesis mean quiz ch test online review final exam</t>
         </is>
       </c>
     </row>
     <row r="193">
       <c r="A193" t="inlineStr">
         <is>
-          <t>STA_2122</t>
+          <t>STA_3033</t>
         </is>
       </c>
       <c r="B193" t="inlineStr">
         <is>
-          <t>sta tr instructor leonid bekker home page http faculty fiu edu bekkerl phone email bekkerl fiu edu office ai office hours mw mw tr course objectives upon successful completion course students able apply working knowledge basic concepts used statistics interpret statistics used journal articles field demonstrate familiarity interpreting output statistical software package build upon foundation work statistics textbook using interactive statistics nd edition michael sullivan iii george woodbury nd mylab mylab guided notebook guided notebook alone students required purchase companion guided notebook interactive statistics exam coverage exam statistical thinking concepts descriptive statistics basic probability chapters exam discrete random variables binomial distribution continuous random variables normal distribution sampling distributions central limit theorem chapters exam confidence intervals hypothesis testing chapters final exam cumulative calculator students may use standard basic scientific calculators drop date march student whose name appears class list date receive letter grade course make policy assignments due indicated unforeseen emergency arises prev ents taking exam documentation must provided e summons jury duty letter physicians letterhead stating explicitly student could hand ass ignment take exam etc course communication contact via canvas mail directly bekkerl fiu edu online assignments include interactive assignments online homework chapter q uizzes chapter exams assigned homework quizzes tests except final exam must completed mystatlab integrated canvas attention proceed next chapter hw previous one accomplished least score prerequisite set every quiz test corresponding chapter hw accomplished least score exams scheduled three online chapter exams cumulative final exam class grading policy course requirements weights interactive assignments online homework quizzes exam exam exam final exam average hw score exceed extra points added final course score following scale basis assigning final grades grade range grade range grade range b c b b c f classroom policies classroom attendance necessary part course students unexcused absences rewarded extra points added final exam score lecture allowed use computers ipads cell phones etc course calendar assignment name date due sections covered introduction ia terminology types data qualitative quantitative types observational studies level measurement hw ia bar graph pie chart shape distribution dot plot histogram quiz ch quiz ch hw ia measures central tendency measures dispersion hw ia percentiles box plots quiz ch hw ia probability sample space union intersection complementary events hw ia additive multiplicative rules conditional probability independent dependent events quiz ch test online hw ia hw discrete random variable binomial random variable ia hw ia poisson random variable quiz ch hw ia continuous random variable normal distribution hw ia quiz ch hw ia sampling distribution mean proportion hw ia confidence interval academic integrity honesty form cheating academic dishonesty strictly forbidden class student found responsible academic misconduct subject academic misconduct procedures sanctions outlined student handbook signature enrolling class agreeing governed po licies syllabus also stating aware syllabus accompanying course calendar schedule subject change needed accommodate unforeseen issues arise term changes announced class posted canvas important read posted announcements daily quiz ch test online ia hw confidence interval proportion population mean hw ia test hypothesis terminology quiz ch hw ia b hw b ia test hypothesis proportion p hw test hypothesis mean quiz ch test online review final exam</t>
+          <t>sta section u class ref course outline introduction probability statistics cs engineering semester spring time pm pm days tu th room gl credit hours prerequisite calculus ii mac equivalence basic knowledge using internet instructor dr h zahedi office dm c phone fax email zahedih fiu edu webpage http faculty fiu edu zahedih blackboard login http online fiu edu login uts html formal office hours mondays tuesday wednesdays thursdays appointments necessary times appointments feel free consult often need whenever problems arise text book probability statistics engineers sheafer mulekar mcclave th edition wadsworth inc coverage objectives cover topics chapters topics ch apters text book plus additional related topics form class notes introductory calculus based undergraduate course basic probability statistics inference computer science engineering majors course intended teach students basic ideas techniques descriptive statistical analysis random even ts probabilities commonly used univariate discrete continuous probability models point estimations interval estimations testing hypotheses commonly used parameters see course syllabus th e second page details assignments weekly homework problems see blackboard list suggested homework proble ms text book supporting materials chapters review problems posted blackboard tentative exams quizzes tbaexam thursday february exam ii thursday march final exam tba register courses final examination conflict course grading quizzes exam exam ii final exam approximate grade scaling b b b c c f policies remarks web assisted course students enrolled course ar e expected fiu email account familiar basics internet u se purpose web based materials c ourse enhance compliment classroom book materials facilitate learning concepts intended substitute classroom lectures expected attend classes regularly exams based materials covered assigned classroom homework assignments web based projects students strongly advised attend lectures time anyone misses exam quiz receive f ex quiz anyone misses final exam receive f course failure hand possible homework assignment time may result reduction points overall grade fail ure complete web based project time may result f grade project make exam given student misses exam due emergency cases meet university quirements student illness loss immediate family member active beepers cellular phones allowed classroom carry make sure switched ff failing student missed classes may receive f instead f academic misconduct florida international university co mmunity dedicated generating impar ting knowledge ex cellent teaching research rigorous respectful exchange ideas community servic e students respect right others n equitable opportunity learn honestly demonstrate quality learning therefore stude nts expected adhere standard academic conduct demonstrates respect fellow students educational mission university students deemed university understand found responsible academic misconduct w ill subject academic misconduct pr ocedures sanctions outlined student handbook following statement required university plagiarism cheating serious offensiv e punishable expulsion university important dates january monday classes beginjanuary monday martin luther king holiday university closed january tuesday last day change grading option last day add courses last day drop courses withdraw university without incurring financial liability tuition fees february friday last day apply graduation end spring term last day withdraw university refund tuition march spring break university open classes march monday last day drop course dr gr ade last day withdraw university wi grade april april final week semester modified cla ss schedule final exams course assessment activities scheduled week may thursday complete grade report available students web information importa nt dates please visit florida intern ational university home page http www fiu edu note course outline subject possible changes case possible changes notified advance sta intro probability statistics cs engineering course syllabus prerequisite calculus ii terms offered fall spring summer text book probability statistics engineers sheaffer mulekar mcclave th ed ition brooks cole cengage learning additional reading needed probability statistics engineering lapin probability statistics engineering com puter sciences j milton j c arnold topics coverage statistics introduction basic ideas tools displaying analyzing data sets approximately weeks probability probability counting rules conditional proba bility independence rules probability approximately weeks discrete probability distributions concepts random variable probability distribution di screte random variable cumulative distribution function mathematical expectation bernoulli distribution binomial dist ribution geometric distribution negative binomial distribution poisson distribution hype rgeometric distribution approximately weeks continuous probability distributions continuous random variable density cumulative distribution functions mathema tical expectation uniform distribution exponential distribution gamma di stribution normal distribution beta distribution weibull di stribution transformations functions random variable probability integral transfor mation theorem application generating simulating random variates given probability distribution approximately weeks statistics sampling distributions sample mean sample variance sampli ng distribution sample mean central li mit theorem normal approximation binomial distribution sampling distribution sample variance approximately week estimation point interval estimators unbiase dness confidence intervals means propor tions variances prediction intervals approximately weeks hypotheses testing testing mean proportion p va riance testing difference two means difference two proport ions paired test testing ratio variances approximately weeks</t>
         </is>
       </c>
     </row>
     <row r="194">
       <c r="A194" t="inlineStr">
         <is>
-          <t>STA_3033</t>
+          <t>STA_4322</t>
         </is>
       </c>
       <c r="B194" t="inlineStr">
         <is>
-          <t>sta section u class ref course outline introduction probability statistics cs engineering semester spring time pm pm days tu th room gl credit hours prerequisite calculus ii mac equivalence basic knowledge using internet instructor dr h zahedi office dm c phone fax email zahedih fiu edu webpage http faculty fiu edu zahedih blackboard login http online fiu edu login uts html formal office hours mondays tuesday wednesdays thursdays appointments necessary times appointments feel free consult often need whenever problems arise text book probability statistics engineers sheafer mulekar mcclave th edition wadsworth inc coverage objectives cover topics chapters topics ch apters text book plus additional related topics form class notes introductory calculus based undergraduate course basic probability statistics inference computer science engineering majors course intended teach students basic ideas techniques descriptive statistical analysis random even ts probabilities commonly used univariate discrete continuous probability models point estimations interval estimations testing hypotheses commonly used parameters see course syllabus th e second page details assignments weekly homework problems see blackboard list suggested homework proble ms text book supporting materials chapters review problems posted blackboard tentative exams quizzes tbaexam thursday february exam ii thursday march final exam tba register courses final examination conflict course grading quizzes exam exam ii final exam approximate grade scaling b b b c c f policies remarks web assisted course students enrolled course ar e expected fiu email account familiar basics internet u se purpose web based materials c ourse enhance compliment classroom book materials facilitate learning concepts intended substitute classroom lectures expected attend classes regularly exams based materials covered assigned classroom homework assignments web based projects students strongly advised attend lectures time anyone misses exam quiz receive f ex quiz anyone misses final exam receive f course failure hand possible homework assignment time may result reduction points overall grade fail ure complete web based project time may result f grade project make exam given student misses exam due emergency cases meet university quirements student illness loss immediate family member active beepers cellular phones allowed classroom carry make sure switched ff failing student missed classes may receive f instead f academic misconduct florida international university co mmunity dedicated generating impar ting knowledge ex cellent teaching research rigorous respectful exchange ideas community servic e students respect right others n equitable opportunity learn honestly demonstrate quality learning therefore stude nts expected adhere standard academic conduct demonstrates respect fellow students educational mission university students deemed university understand found responsible academic misconduct w ill subject academic misconduct pr ocedures sanctions outlined student handbook following statement required university plagiarism cheating serious offensiv e punishable expulsion university important dates january monday classes beginjanuary monday martin luther king holiday university closed january tuesday last day change grading option last day add courses last day drop courses withdraw university without incurring financial liability tuition fees february friday last day apply graduation end spring term last day withdraw university refund tuition march spring break university open classes march monday last day drop course dr gr ade last day withdraw university wi grade april april final week semester modified cla ss schedule final exams course assessment activities scheduled week may thursday complete grade report available students web information importa nt dates please visit florida intern ational university home page http www fiu edu note course outline subject possible changes case possible changes notified advance sta intro probability statistics cs engineering course syllabus prerequisite calculus ii terms offered fall spring summer text book probability statistics engineers sheaffer mulekar mcclave th ed ition brooks cole cengage learning additional reading needed probability statistics engineering lapin probability statistics engineering com puter sciences j milton j c arnold topics coverage statistics introduction basic ideas tools displaying analyzing data sets approximately weeks probability probability counting rules conditional proba bility independence rules probability approximately weeks discrete probability distributions concepts random variable probability distribution di screte random variable cumulative distribution function mathematical expectation bernoulli distribution binomial dist ribution geometric distribution negative binomial distribution poisson distribution hype rgeometric distribution approximately weeks continuous probability distributions continuous random variable density cumulative distribution functions mathema tical expectation uniform distribution exponential distribution gamma di stribution normal distribution beta distribution weibull di stribution transformations functions random variable probability integral transfor mation theorem application generating simulating random variates given probability distribution approximately weeks statistics sampling distributions sample mean sample variance sampli ng distribution sample mean central li mit theorem normal approximation binomial distribution sampling distribution sample variance approximately week estimation point interval estimators unbiase dness confidence intervals means propor tions variances prediction intervals approximately weeks hypotheses testing testing mean proportion p va riance testing difference two means difference two proport ions paired test testing ratio variances approximately weeks</t>
+          <t>course outline sta introduction mathematical statistics ii spring instructor dr golam kibria office dm b phone email kibriag fiu edu web page http faculty fiu edu k ibriag class time place monday wednes day pm pm tba office hours monda wednesday pm pm appointment prerequisite sta introduction mathematical statistics equivalent course text mathematical statistics applications th edition dennis wackerly william mendenhall iii richard l scheaffer cengage learning usa isbn isbn course description second course two semester sequence detailed course outlines presented sampling distribution distribution statistics samp le mean sample variance chi squared f distributions sampling distribution order statistics joint distribution order statistics estimation confidence intervals properties point estimators common unbiased poin estimators evaluating goodness point estimator confidence intervals large sample confidence interval selecting sample size small sample confidence interval properties point estimators method estimation unbiasedness rela tive efficiency consistency minim al sufficiency minimum variance unbiased estimation mvue method moments method maximum likelihood hypothesis testing elements statistical test common large sample tests calculation ype error sample size z test different ways reporting result test attained significance levels p values comments theory hypothesis testing two sample tests based distributions testing hypothesis concerning variances power tests neyman pearson lemma likelihood ratio tests analysis contingency table chi square goodness fit test nonparametric tests sign test signed rank test rank sum tests tests based runs rank correlation linear models estimation least squares optional linear regression estimation least squar es method method least squares connection maximum likelihood method normality assumption confidence intervals parameters prediction interval multiple linear regression analysis variance optional experimental design one way two way analysis variance note scientific calculator required course course evaluation tentativel ighting scheme follows assignments midterm exam midterm exam ii final exam assignments several assignments independently done course ome selected problems assignment graded tentative midterm dates follows first midterm exam held february mon day exam cover materials february wednes day second midterm exam held march mon day exam covers materials march wednes day final exam cumulative exact time date provided soon available ps register class yo ur final exam conflicts course note complain grading midterm exams assignments done within two weeks corresponding exams assignments make exam given however extenuating circum stance exists please contact instructor prior exam receive permission absent must arrange taking substitute test soon possible students required attend final exam failure attend result grade f course unfort unately n extra work given improve grade grading scale weighted average scores three exams converted percentage following scale used assign letter grades course letter range letter range letter range b c b b c f important dates january monday classes begin march last day drop course dr grade last day withdraw university wi grade ps please check university exact date instructor responsible date add drop course etc class end april grades avaliable students thursday april january mon day last day add drop courses withdraw university without incurring financial liability tuition fees january monday martin luther king holiday university closed february monday saturday spring bre ak note instructor responsible date time students must review fiu academic calendar dates instructor responsible add drop course student responsibility incomplete incomplete grade given student completed bulk course works least half course unable complete course due serious interruption caused student negligence choice incomplete grade attendance students expected attend classes regularly student misses fails attend class sole responsibility obtain missing information examples change exam date change exam location add omit sections class notes new home works etc instructor students students encouraged seek instructors help office hours note course outline provides general plan guide course however deviation changes may necessary instructor assume sole authority matters related course content students grading classroom procedur es active beeper cellular phones allowed classes register class final exam conflicts course academic misconduct florida international university community dedicated generating impartin g knowledge excellent teaching research rigorous respectful exchange ideas community service students respect right others equitable opportunity learn honestly demonstrate quality learning therefore students expected adhere standard academic conduct demonstrates respect fellow students educational mission university students deemed university understand found responsible academic misconduct subject academic misconduct procedures sanctions outlined student handbook</t>
         </is>
       </c>
     </row>
     <row r="195">
       <c r="A195" t="inlineStr">
         <is>
-          <t>STA_4322</t>
+          <t>TCN_5010</t>
         </is>
       </c>
       <c r="B195" t="inlineStr">
         <is>
-          <t>course outline sta introduction mathematical statistics ii spring instructor dr golam kibria office dm b phone email kibriag fiu edu web page http faculty fiu edu k ibriag class time place monday wednes day pm pm tba office hours monda wednesday pm pm appointment prerequisite sta introduction mathematical statistics equivalent course text mathematical statistics applications th edition dennis wackerly william mendenhall iii richard l scheaffer cengage learning usa isbn isbn course description second course two semester sequence detailed course outlines presented sampling distribution distribution statistics samp le mean sample variance chi squared f distributions sampling distribution order statistics joint distribution order statistics estimation confidence intervals properties point estimators common unbiased poin estimators evaluating goodness point estimator confidence intervals large sample confidence interval selecting sample size small sample confidence interval properties point estimators method estimation unbiasedness rela tive efficiency consistency minim al sufficiency minimum variance unbiased estimation mvue method moments method maximum likelihood hypothesis testing elements statistical test common large sample tests calculation ype error sample size z test different ways reporting result test attained significance levels p values comments theory hypothesis testing two sample tests based distributions testing hypothesis concerning variances power tests neyman pearson lemma likelihood ratio tests analysis contingency table chi square goodness fit test nonparametric tests sign test signed rank test rank sum tests tests based runs rank correlation linear models estimation least squares optional linear regression estimation least squar es method method least squares connection maximum likelihood method normality assumption confidence intervals parameters prediction interval multiple linear regression analysis variance optional experimental design one way two way analysis variance note scientific calculator required course course evaluation tentativel ighting scheme follows assignments midterm exam midterm exam ii final exam assignments several assignments independently done course ome selected problems assignment graded tentative midterm dates follows first midterm exam held february mon day exam cover materials february wednes day second midterm exam held march mon day exam covers materials march wednes day final exam cumulative exact time date provided soon available ps register class yo ur final exam conflicts course note complain grading midterm exams assignments done within two weeks corresponding exams assignments make exam given however extenuating circum stance exists please contact instructor prior exam receive permission absent must arrange taking substitute test soon possible students required attend final exam failure attend result grade f course unfort unately n extra work given improve grade grading scale weighted average scores three exams converted percentage following scale used assign letter grades course letter range letter range letter range b c b b c f important dates january monday classes begin march last day drop course dr grade last day withdraw university wi grade ps please check university exact date instructor responsible date add drop course etc class end april grades avaliable students thursday april january mon day last day add drop courses withdraw university without incurring financial liability tuition fees january monday martin luther king holiday university closed february monday saturday spring bre ak note instructor responsible date time students must review fiu academic calendar dates instructor responsible add drop course student responsibility incomplete incomplete grade given student completed bulk course works least half course unable complete course due serious interruption caused student negligence choice incomplete grade attendance students expected attend classes regularly student misses fails attend class sole responsibility obtain missing information examples change exam date change exam location add omit sections class notes new home works etc instructor students students encouraged seek instructors help office hours note course outline provides general plan guide course however deviation changes may necessary instructor assume sole authority matters related course content students grading classroom procedur es active beeper cellular phones allowed classes register class final exam conflicts course academic misconduct florida international university community dedicated generating impartin g knowledge excellent teaching research rigorous respectful exchange ideas community service students respect right others equitable opportunity learn honestly demonstrate quality learning therefore students expected adhere standard academic conduct demonstrates respect fellow students educational mission university students deemed university understand found responsible academic misconduct subject academic misconduct procedures sanctions outlined student handbook</t>
+          <t>tcn u telecommunications technology applications spring instructor xuyu wang email xuywang fiu edu place green library lecture time monday pm pm office case office hours monday pm pm zoom link https fiu zoom us j passcode jt qux appointment textbook required text textbook required recommended texts readings computer networking top approach featuring internet rd edition james f kurose keith w ross andrea goldsmith wireless communications cambridge university press new york ny usa wireless communications principles practice theodore rappaport prentice hall course slides assignments artifacts available canvas course content course provides students telecommunication fundamentals emphasis higher level protocols wireless networks applications also course focuses exploiting deep learning methods data networking wireless communications e g signal modulation coding security topics course include state art telecommunication techniques applications e g data networks network iot security edge computing video streaming analysis federated learning wireless systems sensing lte g ai security well next generation telecommunication technologies e g quantum semantic communications satellite networks metaverse course objectives gain breadth depth knowledge data network protocol design develop state art knowledge advanced topics computer networking wireless networks security use deep learning design computer networking wireless networks security provide programming experience telecommunication technology applications tentative schedule subject change week topics major content syllabus introduction ai telecommunication networks martin luther king day class tcp ip review network iot security ai networking edge computing e g video streaming analysis federated learning edge spring break class ai wireless modulation coding wi fi wireless sensing systems wireless iot systems e g lora lte g systems new techniques e g quantum semantic communications new techniques e g satellite oran metaverse ai security pre final review tentative grading policy subject change semester final exam homework assignments project attendance grading breakdown c b f b b c submission rules submission needs electronic version canvas file needs named according one following formats depending submission type please use txt format word pdf format preferable tcn homework name tcn project name example james green submitting project file name submission tcn homework james green first page submitted document please always list name author please note attachment according proper format stated accepted late submission penalized following rules second day submission assignment grade third day submission assignment grade third day assignment grade project two students work together final project policies please review fiu policies webpage policies webpage contains essential information regarding guidelines relevant courses fiu well additional information acceptable netiquette online courses additional information please visit fiu policy procedure library member fiu community expected knowledgeable behavioral expectations set forth fiu student conduct honor code accessibility accommodation disability resource center collaborates students faculty staff community members create diverse learning environments usable equitable inclusive sustainable drc provides fiu students disabilities necessary support successfully complete education participate activities available students diagnosed disability plan utilize academic accommodations please contact center visit graham center gc additional assistance please contact fiu disability resource center please visit ada compliance webpage additional information accessibility involving tools used course academic misconduct statement florida international university community dedicated generating imparting knowledge excellent teaching research rigorous respectful exchange ideas community service students respect right others equitable opportunity learn honestly demonstrate quality learning therefore students expected adhere standard academic conduct demonstrates respect fellow students educational mission university students deemed university understand found responsible academic misconduct subject academic misconduct procedures sanctions outlined student conduct honor code academic misconduct includes cheating unauthorized use materials information study aids assistance another person academic assignment exercise unless explicitly authorized course instructor assisting another student unauthorized use materials information study aids unless explicitly authorized instructor substitute complete academic assignment completing academic assignment someone else either paid unpaid plagiarism deliberate use appropriation another work without indication source representation work student assisting another student deliberate use appropriation another work without indication source representation work student learn academic integrity policies procedures well student resources help prepare successful semester panthers care counseling psychological services caps looking help fellow classmate panthers care encourages express concerns may come across relates personal behavior concerns worries classmate well encouraged share concerns fiu panthers care website counseling psychological services caps offers free confidential help anxiety depression stress concerns life brings professional counselors available day appointments wait call set time talk visit online self help portal</t>
         </is>
       </c>
     </row>
     <row r="196">
       <c r="A196" t="inlineStr">
         <is>
-          <t>TCN_5010</t>
+          <t>TCN_5030</t>
         </is>
       </c>
       <c r="B196" t="inlineStr">
         <is>
-          <t>tcn u telecommunications technology applications spring instructor xuyu wang email xuywang fiu edu place green library lecture time monday pm pm office case office hours monday pm pm zoom link https fiu zoom us j passcode jt qux appointment textbook required text textbook required recommended texts readings computer networking top approach featuring internet rd edition james f kurose keith w ross andrea goldsmith wireless communications cambridge university press new york ny usa wireless communications principles practice theodore rappaport prentice hall course slides assignments artifacts available canvas course content course provides students telecommunication fundamentals emphasis higher level protocols wireless networks applications also course focuses exploiting deep learning methods data networking wireless communications e g signal modulation coding security topics course include state art telecommunication techniques applications e g data networks network iot security edge computing video streaming analysis federated learning wireless systems sensing lte g ai security well next generation telecommunication technologies e g quantum semantic communications satellite networks metaverse course objectives gain breadth depth knowledge data network protocol design develop state art knowledge advanced topics computer networking wireless networks security use deep learning design computer networking wireless networks security provide programming experience telecommunication technology applications tentative schedule subject change week topics major content syllabus introduction ai telecommunication networks martin luther king day class tcp ip review network iot security ai networking edge computing e g video streaming analysis federated learning edge spring break class ai wireless modulation coding wi fi wireless sensing systems wireless iot systems e g lora lte g systems new techniques e g quantum semantic communications new techniques e g satellite oran metaverse ai security pre final review tentative grading policy subject change semester final exam homework assignments project attendance grading breakdown c b f b b c submission rules submission needs electronic version canvas file needs named according one following formats depending submission type please use txt format word pdf format preferable tcn homework name tcn project name example james green submitting project file name submission tcn homework james green first page submitted document please always list name author please note attachment according proper format stated accepted late submission penalized following rules second day submission assignment grade third day submission assignment grade third day assignment grade project two students work together final project policies please review fiu policies webpage policies webpage contains essential information regarding guidelines relevant courses fiu well additional information acceptable netiquette online courses additional information please visit fiu policy procedure library member fiu community expected knowledgeable behavioral expectations set forth fiu student conduct honor code accessibility accommodation disability resource center collaborates students faculty staff community members create diverse learning environments usable equitable inclusive sustainable drc provides fiu students disabilities necessary support successfully complete education participate activities available students diagnosed disability plan utilize academic accommodations please contact center visit graham center gc additional assistance please contact fiu disability resource center please visit ada compliance webpage additional information accessibility involving tools used course academic misconduct statement florida international university community dedicated generating imparting knowledge excellent teaching research rigorous respectful exchange ideas community service students respect right others equitable opportunity learn honestly demonstrate quality learning therefore students expected adhere standard academic conduct demonstrates respect fellow students educational mission university students deemed university understand found responsible academic misconduct subject academic misconduct procedures sanctions outlined student conduct honor code academic misconduct includes cheating unauthorized use materials information study aids assistance another person academic assignment exercise unless explicitly authorized course instructor assisting another student unauthorized use materials information study aids unless explicitly authorized instructor substitute complete academic assignment completing academic assignment someone else either paid unpaid plagiarism deliberate use appropriation another work without indication source representation work student assisting another student deliberate use appropriation another work without indication source representation work student learn academic integrity policies procedures well student resources help prepare successful semester panthers care counseling psychological services caps looking help fellow classmate panthers care encourages express concerns may come across relates personal behavior concerns worries classmate well encouraged share concerns fiu panthers care website counseling psychological services caps offers free confidential help anxiety depression stress concerns life brings professional counselors available day appointments wait call set time talk visit online self help portal</t>
+          <t>tcn computer communications networking technologies catalog description teaches dynamics related computer communications computers grouped together form networks various networ king implementation strategies current technologies credits prerequisites scis graduate standing type required mstn course objectives course provides introduction th e concepts principles computer communications networks students un derstand architectures protocols techniques different layers internet protocol stack addition students learn fundamental network progr amming analyzing skills topics introduction application layer transport layer network layer link layer local area networks multimedia networking network management textbook james kurose keith ross computer networking top approach th edition addison wesley larry peterson bruce davie computer ne tworks systems approach th edition morgan kaufmann andrew tanenbaum comput er networks th edition prentice hall last update deng pan</t>
         </is>
       </c>
     </row>
     <row r="197">
       <c r="A197" t="inlineStr">
         <is>
-          <t>TCN_5030</t>
+          <t>TCN_5060</t>
         </is>
       </c>
       <c r="B197" t="inlineStr">
         <is>
-          <t>tcn computer communications networking technologies catalog description teaches dynamics related computer communications computers grouped together form networks various networ king implementation strategies current technologies credits prerequisites scis graduate standing type required mstn course objectives course provides introduction th e concepts principles computer communications networks students un derstand architectures protocols techniques different layers internet protocol stack addition students learn fundamental network progr amming analyzing skills topics introduction application layer transport layer network layer link layer local area networks multimedia networking network management textbook james kurose keith ross computer networking top approach th edition addison wesley larry peterson bruce davie computer ne tworks systems approach th edition morgan kaufmann andrew tanenbaum comput er networks th edition prentice hall last update deng pan</t>
+          <t>tcn u telecommunications software methodologies spring term instructor name mo sha knight foundation school computing information sciences florida international university email msha fiu edu phone office case office hours th zoom zoom link https fiu zoom us j appointment tentative class schedule course description purpose course provides students high level look network architectures distributed applications client server models network software platforms advanced techniques programs specifications implementation substantial part material cover telecommunications systems wireless networks embedded operating systems network protocols variety different telecommunications applications introduced including clinical monitoring structural health monitoring industrial process automation course students also opportunity obt hands experience programming embedded devices sense communicate please visit course website details course objectives learning outcomes upon completi ng course students able identify telecommunications devices identify major telecommunications applications understand basic concepts features embedded operating systems understand characteristics constraints wireless communi cation frequency bands modulation signal distortion interference compare different medium access control protocols understand basic concepts telecommunications techniques create telecommunications applications using embedded programming language important information starting course please review following pages accessibility accommodation academic misconduct statement professor retains right modify course syllabus reason throughout semester prerequisites corequisites none textbook required reference books philip levis david gay tinyos programming cambridge university press isbn free download main topics following topics covered may covered partially main topics topic introduction telecommunications embedded operating systems tinyos android programming language networked embedded systems wireless protocol stack physical layer wireless protocol stack mac layer wireless protocol stack routing layer introduction machine learning telecommunications applications clinical monitoring telecommunications applications structural health monitoring telecommunications applications industrial process automation advanced topics time permits lecture slides supplemental materials lecture slides posted module canvas lecture take notes class compare lecture slides posted ensure understand concepts presented lecture slides substitute class attendance beca use complete ii significant parts lectures including discussions class exercises may come lecture slides additional materials added appropriate assignments one programming assignment ssignment lead implementation basic telecommunications application requires understanding application concepts designs introduced class student required complete assignment independently three pape r presentations one semester long system project project lead implementation complete telecommunications system solves real world problem identified student project individual project spend lo time project class class start working project early know solve problem give talk instructor classmate readability programs solutions necessary correctness expect lose points provide badly written unclear correct solution code well commented late submissions accepted circumstances plan turn required project documents early grading scheme following percentage weights used assess student work programming assignment paper presentations project reference approximate breakdown grades previous class approximate breakdown grades previous class letter range letter range letter range b c b b c f less academic integrity expectations florida international university community dedicated generating imparting knowledge excellent teaching research rigorous respectful exchange ideas community service students respect righ others equitable opportunity learn honestly demonstrate quality learning therefore students expected adhere standard academic conduct demonstrates respect fellow stude nts educational mission university students deemed university understand found responsible academic misconduct subject student conduct honor code procedures sanctions utlined fiu regulation student handbook please review student conduct academic integrity website academi c misconduct statement make sure understand programming assignment submission must following statement done assignment completely copied given solution anyone else understand involved plagiarism cheating receive penalty specified fiu regulations collaboration assignment students encouraged help one another form study groups computer science lear n peers instructors teaching assistants long help appropriate please generous time expertise helping fellow students good good free discuss assignment general terms one another however please show work directly students student must complete assignments individually unless indicated otherwise instructor must write code must write solutions individually students submitting solutions including code determined similar likely punished equally harshly tell whether done work please work disability resource center disability resource center drc collaborates university faculty provide inclusive learning environments disability plan utilize academic accommodations additional informa tion may found drc website panthers cares caps services looking help fellow classmate panthers care encourages express concerns may come acros relates personal behavior concerns worries classmate well encouraged share concerns fiu panthers care website counseling psychological services caps offers free confidential help anxiety depression stress concerns life brings learn caps caps fiu edu professional counselors availa ble day appointments wait call set time talk visit online self help portal intellectual property rights student work submitted college school department satisfaction course degree requirements becomes physical property college school department work may include papers drawings models materials however students retain rights intellectual property work created part academic course may request upon completion academic course college school department return work student holding intellectual property rights therein student declines accept physical possession student work college school department may discretion retain return discard materials college school departm ent normally discard materials currently enrolled students college school department wishes use student work request student voluntarily consent writing use consent given college schoo l department include student name using student work please advised classes may audio visually recorded subject course capture future access students course attendance participation course constitutes consent recordings used educational purposes students course securely stored university systems concern regarding recording use recording please contact ferpa fiu edu class attendance requirement attendance required attendance checked regularly present attendance checked counted missing class may miss total three classes without verifiable valid excuse final grad e reduced missing class miss six additional beyond three classes automatically fail class please inform instructor ahead time email expected excused absence may make cla ss attending section computers electronic devices allowed use phone laptop notebook tablet class unless explicitly permitted cell phones must turned vibrate alert mode class</t>
         </is>
       </c>
     </row>
     <row r="198">
       <c r="A198" t="inlineStr">
         <is>
-          <t>TCN_5060</t>
+          <t>TCN_5080</t>
         </is>
       </c>
       <c r="B198" t="inlineStr">
         <is>
-          <t>tcn u telecommunications software methodologies spring term instructor name mo sha knight foundation school computing information sciences florida international university email msha fiu edu phone office case office hours th zoom zoom link https fiu zoom us j appointment tentative class schedule course description purpose course provides students high level look network architectures distributed applications client server models network software platforms advanced techniques programs specifications implementation substantial part material cover telecommunications systems wireless networks embedded operating systems network protocols variety different telecommunications applications introduced including clinical monitoring structural health monitoring industrial process automation course students also opportunity obt hands experience programming embedded devices sense communicate please visit course website details course objectives learning outcomes upon completi ng course students able identify telecommunications devices identify major telecommunications applications understand basic concepts features embedded operating systems understand characteristics constraints wireless communi cation frequency bands modulation signal distortion interference compare different medium access control protocols understand basic concepts telecommunications techniques create telecommunications applications using embedded programming language important information starting course please review following pages accessibility accommodation academic misconduct statement professor retains right modify course syllabus reason throughout semester prerequisites corequisites none textbook required reference books philip levis david gay tinyos programming cambridge university press isbn free download main topics following topics covered may covered partially main topics topic introduction telecommunications embedded operating systems tinyos android programming language networked embedded systems wireless protocol stack physical layer wireless protocol stack mac layer wireless protocol stack routing layer introduction machine learning telecommunications applications clinical monitoring telecommunications applications structural health monitoring telecommunications applications industrial process automation advanced topics time permits lecture slides supplemental materials lecture slides posted module canvas lecture take notes class compare lecture slides posted ensure understand concepts presented lecture slides substitute class attendance beca use complete ii significant parts lectures including discussions class exercises may come lecture slides additional materials added appropriate assignments one programming assignment ssignment lead implementation basic telecommunications application requires understanding application concepts designs introduced class student required complete assignment independently three pape r presentations one semester long system project project lead implementation complete telecommunications system solves real world problem identified student project individual project spend lo time project class class start working project early know solve problem give talk instructor classmate readability programs solutions necessary correctness expect lose points provide badly written unclear correct solution code well commented late submissions accepted circumstances plan turn required project documents early grading scheme following percentage weights used assess student work programming assignment paper presentations project reference approximate breakdown grades previous class approximate breakdown grades previous class letter range letter range letter range b c b b c f less academic integrity expectations florida international university community dedicated generating imparting knowledge excellent teaching research rigorous respectful exchange ideas community service students respect righ others equitable opportunity learn honestly demonstrate quality learning therefore students expected adhere standard academic conduct demonstrates respect fellow stude nts educational mission university students deemed university understand found responsible academic misconduct subject student conduct honor code procedures sanctions utlined fiu regulation student handbook please review student conduct academic integrity website academi c misconduct statement make sure understand programming assignment submission must following statement done assignment completely copied given solution anyone else understand involved plagiarism cheating receive penalty specified fiu regulations collaboration assignment students encouraged help one another form study groups computer science lear n peers instructors teaching assistants long help appropriate please generous time expertise helping fellow students good good free discuss assignment general terms one another however please show work directly students student must complete assignments individually unless indicated otherwise instructor must write code must write solutions individually students submitting solutions including code determined similar likely punished equally harshly tell whether done work please work disability resource center disability resource center drc collaborates university faculty provide inclusive learning environments disability plan utilize academic accommodations additional informa tion may found drc website panthers cares caps services looking help fellow classmate panthers care encourages express concerns may come acros relates personal behavior concerns worries classmate well encouraged share concerns fiu panthers care website counseling psychological services caps offers free confidential help anxiety depression stress concerns life brings learn caps caps fiu edu professional counselors availa ble day appointments wait call set time talk visit online self help portal intellectual property rights student work submitted college school department satisfaction course degree requirements becomes physical property college school department work may include papers drawings models materials however students retain rights intellectual property work created part academic course may request upon completion academic course college school department return work student holding intellectual property rights therein student declines accept physical possession student work college school department may discretion retain return discard materials college school departm ent normally discard materials currently enrolled students college school department wishes use student work request student voluntarily consent writing use consent given college schoo l department include student name using student work please advised classes may audio visually recorded subject course capture future access students course attendance participation course constitutes consent recordings used educational purposes students course securely stored university systems concern regarding recording use recording please contact ferpa fiu edu class attendance requirement attendance required attendance checked regularly present attendance checked counted missing class may miss total three classes without verifiable valid excuse final grad e reduced missing class miss six additional beyond three classes automatically fail class please inform instructor ahead time email expected excused absence may make cla ss attending section computers electronic devices allowed use phone laptop notebook tablet class unless explicitly permitted cell phones must turned vibrate alert mode class</t>
+          <t>tcn secure telecommunications transactions catalog description telecom information security issues su ch digital signatu res cryptography applied telecom transactions network po licing nested authenti cation improving system trust credits prerequisites tcn permission instructor type required mstn course objectives course provides depth unders tanding threats principles mechanisms network security students study cryptographic algorithms applications security prot ocols different layers internet protocol stack students also learn determine appr opriate security mechanisms specific network applications topics symmetric key encryption public key encryption hash functions message authentication code digital signatures authentication protocols ip security email security web security firewalls textbook charlie kaufman radia perlman mike speciner network security private communication public worl nd edition prentice hall william stallings cryptography network security th edition prentice hall matt bishop introduction computer security addison wesley last update deng pan</t>
         </is>
       </c>
     </row>
     <row r="199">
       <c r="A199" t="inlineStr">
         <is>
-          <t>TCN_5080</t>
+          <t>TCN_5421</t>
         </is>
       </c>
       <c r="B199" t="inlineStr">
         <is>
-          <t>tcn secure telecommunications transactions catalog description telecom information security issues su ch digital signatu res cryptography applied telecom transactions network po licing nested authenti cation improving system trust credits prerequisites tcn permission instructor type required mstn course objectives course provides depth unders tanding threats principles mechanisms network security students study cryptographic algorithms applications security prot ocols different layers internet protocol stack students also learn determine appr opriate security mechanisms specific network applications topics symmetric key encryption public key encryption hash functions message authentication code digital signatures authentication protocols ip security email security web security firewalls textbook charlie kaufman radia perlman mike speciner network security private communication public worl nd edition prentice hall william stallings cryptography network security th edition prentice hall matt bishop introduction computer security addison wesley last update deng pan</t>
+          <t>tcn theory ne tworked computation catalog description fundamental mathematical models genera l networked computation finite state automata regular languages decidability st ochastic processes markov chains queueing theory credits prerequisites scis graduate standing type elective mstn core option phd course objectives course provides depth understa nding theore tical foundations networked computation addition various models general computation finite state automata decidability theo ry students also learn mathematical background stochastic pro cesses queueing models topics introduction finite state automata regular languages decidability random variables stochastic processes markov chains queueing analysis computer systems textbook michael sipser introduction theory computation rd edition course technology gross j shortle j thompson c harris fundamentals queueing theory th edition wiley last update deng pan shaolei ren</t>
         </is>
       </c>
     </row>
     <row r="200">
       <c r="A200" t="inlineStr">
         <is>
-          <t>TCN_5421</t>
+          <t>TCN_5440</t>
         </is>
       </c>
       <c r="B200" t="inlineStr">
         <is>
-          <t>tcn theory ne tworked computation catalog description fundamental mathematical models genera l networked computation finite state automata regular languages decidability st ochastic processes markov chains queueing theory credits prerequisites scis graduate standing type elective mstn core option phd course objectives course provides depth understa nding theore tical foundations networked computation addition various models general computation finite state automata decidability theo ry students also learn mathematical background stochastic pro cesses queueing models topics introduction finite state automata regular languages decidability random variables stochastic processes markov chains queueing analysis computer systems textbook michael sipser introduction theory computation rd edition course technology gross j shortle j thompson c harris fundamentals queueing theory th edition wiley last update deng pan shaolei ren</t>
+          <t>tcn u software development telecommunication networks fall term instructor name mo sha knight foundation school computing information sciences florida international university email msha fiu edu phone office case office hours th pm zoom zoom link https fiu zoom us j appointment please email one session want attend office hours tentative class schedule course description purpose telecommunication networks provide basis internet things enable many new applications smart home smart healthcare smart city course focuses aspects tools techniques developing software applications telecommunications networks substantial part material cover programming linux environment programming telecommunication networ ks wireless networks course introduce variety programming concepts software development techniques help students improve programming skills course students opportunities obtain hands experience n programming software development telecommunication networks please visit course website details course objectives learning outcomes upon completing cou rse students able understand basic concepts fundamental features telecommunication networks understand key programming concepts problem solving techniques program linux environment without th e help integrated development environment ide program solve problems using c networked embedded system c nesc languages implement simple data structures develop software sensing communication understand key characteristics constraints wireless networks important information starting course please review following pages accessibility accommodation academic misconduct statement professor retains right modify course syllabus reason throughout semester prerequisites corequisites none textbook required reference books brian w kernighan dennis ritchie c programming language rd edition prentice hall free download online philip levis david gay tinyos programming cambridge university press isbn free download main topics following topics co vered may covered partially main topic introduction telecommunication networks c programming language programming linux environment programming concepts problem solving techniques implementations simple data structures networked embedded system c nesc language programming sensing communication embedded devices advanced topics time permits lecture slides supplemental materials lecture slides posted module canvas lecture take notes class compare lecture slides posted ensure understand concepts presented lecture slides substitute class attendance complete ii significant parts lectures including discussions class exercises may come lecture slides additional materials added appropriate grading scheme following percentage weights used assess student work programming assignment quizzes reference approximate breakdown grades previous class approximate brea kdown grades previous class letter range letter range letter range b c b b c f less programming assignment several programming assignments assignment requires understanding application concepts designs introduced class student required complete assignment independently know implement assignment give please talk instructor readability implementation necessary correctness expect lose points provide badly written unclear correct solution c ode well commented late submissions accepted circumstances plan turn submission early quizzes three class quizzes programming software development quizzes class closed notes clos ed book must take quiz one time give give makeup quizzes academic integrity expectations florida international university community dedicated generating imparting knowledge excellent teachin g research rigorous respectful exchange ideas community service students respect right others equitable opportunity learn honestly demonstrate quality learning therefore studen ts expected adhere standard academic conduct demonstrates respect fellow students educational mission university students deemed university understand found res ponsible academic misconduct subject student conduct honor code procedures sanctions outlined fiu regulation student handbook please review student conduct academic inte grity website academic misconduct statement make sure understand programming assignment submission must f ollowing statement done assignment completely copied given solution anyone else understand involved plagiarism cheating receive penalty specified fiu regulatio ns collaboration assignment students encouraged help one another form study groups computer science learn peers instructors teaching assistants long help appropriate please b e generous time expertise helping fellow students good good free discuss assignment general terms one another however please show work directly students ea ch student must complete assignments individually unless indicated otherwise instructor must write code must write solutions individually students submitting solutions including code determine similar likely punished equally harshly tell whether done work please work disability resource center disability resource center drc collaborates university fac ulty provide inclusive learning environments disability plan utilize academic accommodations additional information may found drc website panthers cares caps service looking help fellow classmate panthers care encourages express concerns may come across relates personal behavior concerns worries classmate well e ncouraged share concerns fiu panthers care website counseling psychological services caps offers free confidential help anxiety depression stress concerns hat life brings learn caps caps fiu edu professional counselors available day appointments wait call set time talk visit online self help portal intellectual property rights student work submitted college school department satisfaction course degree requirements becomes physical property college school department work may include papers drawings models materials however students retain rights intellectual property work created part academic course may request upon completion academic course college school department return work student holding intellectual property rights therein student declines accept physical possession st udent work college school department may discretion retain return discard materials college school department normally discard materials currently enrolled students college school department wishes use student work request student voluntarily consent writing use consent given college school department include student name using student work please advised classes may audio nd visually recorded subject course capture future access students course attendance participation course constitutes consent recordings used educational purposes students co urse securely stored university systems concern regarding recording use recording please contact ferpa fiu edu class attendance requirement attendance required attendance checked regularly present attendance checked counted missing class may miss total three classes without verifiable valid excuse final grade reduced missing class miss six addi tional beyond three classes automatically fail class please inform instructor ahead time email expected excused absence may make class performing activities computers electronic devices allowed use phone laptop notebook tablet class unless explicitly permitted cell phones must turned vibrate alert mode class</t>
         </is>
       </c>
     </row>
     <row r="201">
       <c r="A201" t="inlineStr">
         <is>
-          <t>TCN_5440</t>
+          <t>TCN_5445</t>
         </is>
       </c>
       <c r="B201" t="inlineStr">
         <is>
-          <t>tcn u software development telecommunication networks fall term instructor name mo sha knight foundation school computing information sciences florida international university email msha fiu edu phone office case office hours th pm zoom zoom link https fiu zoom us j appointment please email one session want attend office hours tentative class schedule course description purpose telecommunication networks provide basis internet things enable many new applications smart home smart healthcare smart city course focuses aspects tools techniques developing software applications telecommunications networks substantial part material cover programming linux environment programming telecommunication networ ks wireless networks course introduce variety programming concepts software development techniques help students improve programming skills course students opportunities obtain hands experience n programming software development telecommunication networks please visit course website details course objectives learning outcomes upon completing cou rse students able understand basic concepts fundamental features telecommunication networks understand key programming concepts problem solving techniques program linux environment without th e help integrated development environment ide program solve problems using c networked embedded system c nesc languages implement simple data structures develop software sensing communication understand key characteristics constraints wireless networks important information starting course please review following pages accessibility accommodation academic misconduct statement professor retains right modify course syllabus reason throughout semester prerequisites corequisites none textbook required reference books brian w kernighan dennis ritchie c programming language rd edition prentice hall free download online philip levis david gay tinyos programming cambridge university press isbn free download main topics following topics co vered may covered partially main topic introduction telecommunication networks c programming language programming linux environment programming concepts problem solving techniques implementations simple data structures networked embedded system c nesc language programming sensing communication embedded devices advanced topics time permits lecture slides supplemental materials lecture slides posted module canvas lecture take notes class compare lecture slides posted ensure understand concepts presented lecture slides substitute class attendance complete ii significant parts lectures including discussions class exercises may come lecture slides additional materials added appropriate grading scheme following percentage weights used assess student work programming assignment quizzes reference approximate breakdown grades previous class approximate brea kdown grades previous class letter range letter range letter range b c b b c f less programming assignment several programming assignments assignment requires understanding application concepts designs introduced class student required complete assignment independently know implement assignment give please talk instructor readability implementation necessary correctness expect lose points provide badly written unclear correct solution c ode well commented late submissions accepted circumstances plan turn submission early quizzes three class quizzes programming software development quizzes class closed notes clos ed book must take quiz one time give give makeup quizzes academic integrity expectations florida international university community dedicated generating imparting knowledge excellent teachin g research rigorous respectful exchange ideas community service students respect right others equitable opportunity learn honestly demonstrate quality learning therefore studen ts expected adhere standard academic conduct demonstrates respect fellow students educational mission university students deemed university understand found res ponsible academic misconduct subject student conduct honor code procedures sanctions outlined fiu regulation student handbook please review student conduct academic inte grity website academic misconduct statement make sure understand programming assignment submission must f ollowing statement done assignment completely copied given solution anyone else understand involved plagiarism cheating receive penalty specified fiu regulatio ns collaboration assignment students encouraged help one another form study groups computer science learn peers instructors teaching assistants long help appropriate please b e generous time expertise helping fellow students good good free discuss assignment general terms one another however please show work directly students ea ch student must complete assignments individually unless indicated otherwise instructor must write code must write solutions individually students submitting solutions including code determine similar likely punished equally harshly tell whether done work please work disability resource center disability resource center drc collaborates university fac ulty provide inclusive learning environments disability plan utilize academic accommodations additional information may found drc website panthers cares caps service looking help fellow classmate panthers care encourages express concerns may come across relates personal behavior concerns worries classmate well e ncouraged share concerns fiu panthers care website counseling psychological services caps offers free confidential help anxiety depression stress concerns hat life brings learn caps caps fiu edu professional counselors available day appointments wait call set time talk visit online self help portal intellectual property rights student work submitted college school department satisfaction course degree requirements becomes physical property college school department work may include papers drawings models materials however students retain rights intellectual property work created part academic course may request upon completion academic course college school department return work student holding intellectual property rights therein student declines accept physical possession st udent work college school department may discretion retain return discard materials college school department normally discard materials currently enrolled students college school department wishes use student work request student voluntarily consent writing use consent given college school department include student name using student work please advised classes may audio nd visually recorded subject course capture future access students course attendance participation course constitutes consent recordings used educational purposes students co urse securely stored university systems concern regarding recording use recording please contact ferpa fiu edu class attendance requirement attendance required attendance checked regularly present attendance checked counted missing class may miss total three classes without verifiable valid excuse final grade reduced missing class miss six addi tional beyond three classes automatically fail class please inform instructor ahead time email expected excused absence may make class performing activities computers electronic devices allowed use phone laptop notebook tablet class unless explicitly permitted cell phones must turned vibrate alert mode class</t>
+          <t>tcn telecommunication network programming catalog description advanced telecommunications network programming skills including router bridge software socket programming protocol handler credits prerequisites scis graduate standing type elective mstn core option phd course objectives course teaches network programming system perspective uses unix linux example provides stud ents essential network system programming skill training addition sock et programming student also learn depth system fundamentals including multi threading ipc synchronization shared memory topics introduction tcp udp socket programming multiplexing name address conversions daemon processes inetd superserver nonblocking routing sockets broadcasting multicasting multi threading interprocess communication synchronization mutexes semaphores shared memory remote procedure calls textbook w richard stevens bill fenner ndrew rudoff unix network programming volume sockets networking api rd edition addison wesley professional w richard stevens unix network pr ogramming volume interprocess communications nd edition prentice hall last update deng pan</t>
         </is>
       </c>
     </row>
     <row r="202">
       <c r="A202" t="inlineStr">
         <is>
-          <t>TCN_5445</t>
+          <t>TCN_5455</t>
         </is>
       </c>
       <c r="B202" t="inlineStr">
         <is>
-          <t>tcn telecommunication network programming catalog description advanced telecommunications network programming skills including router bridge software socket programming protocol handler credits prerequisites scis graduate standing type elective mstn core option phd course objectives course teaches network programming system perspective uses unix linux example provides stud ents essential network system programming skill training addition sock et programming student also learn depth system fundamentals including multi threading ipc synchronization shared memory topics introduction tcp udp socket programming multiplexing name address conversions daemon processes inetd superserver nonblocking routing sockets broadcasting multicasting multi threading interprocess communication synchronization mutexes semaphores shared memory remote procedure calls textbook w richard stevens bill fenner ndrew rudoff unix network programming volume sockets networking api rd edition addison wesley professional w richard stevens unix network pr ogramming volume interprocess communications nd edition prentice hall last update deng pan</t>
+          <t>tcn information theory catalog description entropy measures information proof interpretation shannon source channel coding theorems prerequisites permission instructor course objectives course covers topics classical information theory including modeling quanti cation infor mation asymptotic equipartition property data compression channel coding lossy source coding rate distortion theory brief overview kolmogorov complexity topics information measures entropy relative entropy mutual information asymptotic equipartition property entropy rates stochastic processes modeling sources information lossless source encoding theorems source coding techniques data compression di erential entropy gaussian data compression transmission lossy source coding rate distortion theory kolmogorov complexity textbook course material tm cover ja thomas elements information theory nd edition john wiley sons rg gallager information theory reliable communication vol new york wiley csiszar j k orner information theory coding theorems discrete memoryless systems cam bridge university press last updated farhad shirani page</t>
         </is>
       </c>
     </row>
     <row r="203">
       <c r="A203" t="inlineStr">
         <is>
-          <t>TCN_5455</t>
+          <t>TCN_5640</t>
         </is>
       </c>
       <c r="B203" t="inlineStr">
         <is>
-          <t>tcn information theory catalog description entropy measures information proof interpretation shannon source channel coding theorems prerequisites permission instructor course objectives course covers topics classical information theory including modeling quanti cation infor mation asymptotic equipartition property data compression channel coding lossy source coding rate distortion theory brief overview kolmogorov complexity topics information measures entropy relative entropy mutual information asymptotic equipartition property entropy rates stochastic processes modeling sources information lossless source encoding theorems source coding techniques data compression di erential entropy gaussian data compression transmission lossy source coding rate distortion theory kolmogorov complexity textbook course material tm cover ja thomas elements information theory nd edition john wiley sons rg gallager information theory reliable communication vol new york wiley csiszar j k orner information theory coding theorems discrete memoryless systems cam bridge university press last updated farhad shirani page</t>
+          <t>tcn telecommunications enterprise planning strategy catalog description methodologies engineer ing project management strategic planning change management rfps life cycle management within telecommunications arena prerequisites graduate standing permission instructor type required mstn course objectives course examines theory practice telecommunications en terprise planning strategy processes learning outcomes include familiarity essential requirements successful planning new teleco mmunications ne tworking venture essential requirements developmen successful telecommunications networking new venture plan topics overview telecommunications industr changes actors telecom industry strategy telecom entrepreneurial companies telecom product development developing telecom business plan telecom market analysis segmentation planning telecom product cycle assessing telecom technology ventures evaluating telecom business plans legal issues corporate governance fundamentals inte llectual property case studies textbook assigned required recommended reading material assigned class website students responsible fo r using uniform resource location url addresses provided website locate assigned material course syllabus web links assigned reading material last update dr niki pissinou</t>
         </is>
       </c>
     </row>
     <row r="204">
       <c r="A204" t="inlineStr">
         <is>
-          <t>TCN_5640</t>
+          <t>TCN_6215</t>
         </is>
       </c>
       <c r="B204" t="inlineStr">
         <is>
-          <t>tcn telecommunications enterprise planning strategy catalog description methodologies engineer ing project management strategic planning change management rfps life cycle management within telecommunications arena prerequisites graduate standing permission instructor type required mstn course objectives course examines theory practice telecommunications en terprise planning strategy processes learning outcomes include familiarity essential requirements successful planning new teleco mmunications ne tworking venture essential requirements developmen successful telecommunications networking new venture plan topics overview telecommunications industr changes actors telecom industry strategy telecom entrepreneurial companies telecom product development developing telecom business plan telecom market analysis segmentation planning telecom product cycle assessing telecom technology ventures evaluating telecom business plans legal issues corporate governance fundamentals inte llectual property case studies textbook assigned required recommended reading material assigned class website students responsible fo r using uniform resource location url addresses provided website locate assigned material course syllabus web links assigned reading material last update dr niki pissinou</t>
+          <t>tcn advanced network algorithms catalog description course cover algorithms us ed network research implementation credits prerequisites scis graduate standing type elective mstn course objectives students study advanced network algorithms lve research problems implementation challenges students learn design efficient practical algorithms specific problems wired wireless networks topics graph theory computational geometry maximum flow combinatorial optimization np completeness queuing theory fair queuing algorithms switch scheduling algorithms textbook thomas cormen charles leiserson ronald rivest clifford stein introduction algorithms rd edition mit press steve skiena algorithm design manual nd edition springer last update deng pan</t>
         </is>
       </c>
     </row>
     <row r="205">
       <c r="A205" t="inlineStr">
         <is>
-          <t>TCN_6215</t>
+          <t>TCN_6260</t>
         </is>
       </c>
       <c r="B205" t="inlineStr">
         <is>
-          <t>tcn advanced network algorithms catalog description course cover algorithms us ed network research implementation credits prerequisites scis graduate standing type elective mstn course objectives students study advanced network algorithms lve research problems implementation challenges students learn design efficient practical algorithms specific problems wired wireless networks topics graph theory computational geometry maximum flow combinatorial optimization np completeness queuing theory fair queuing algorithms switch scheduling algorithms textbook thomas cormen charles leiserson ronald rivest clifford stein introduction algorithms rd edition mit press steve skiena algorithm design manual nd edition springer last update deng pan</t>
+          <t>tcn internetworking catalog description course discuss advanced topics curre nt trends control internetworking analytical descriptive approach used cover subject internetworking credits prerequisites scis graduate standing type elective mstn course objectives course provides depth understand ing internetwork ing techniques current internet students study vari ous routing switching algorithms protocols including tra inter routing router switc h architecture switch scheduling traffic engineering students also learn hands operation typical routers switches topics introduction routing algorithms network flow optimization routing protocols ip address lookup packet classification switch architecture packet queuing scheduling traffic conditioning textbook deepankar medhi karthikeyan ramasamy network routing algorithms protocols architectures morgan kaufmann h jonathan chao bin liu high perfor mance switches routers wiley ieee press last update deng pan</t>
         </is>
       </c>
     </row>
     <row r="206">
       <c r="A206" t="inlineStr">
         <is>
-          <t>TCN_6260</t>
+          <t>TCN_6270</t>
         </is>
       </c>
       <c r="B206" t="inlineStr">
         <is>
-          <t>tcn internetworking catalog description course discuss advanced topics curre nt trends control internetworking analytical descriptive approach used cover subject internetworking credits prerequisites scis graduate standing type elective mstn course objectives course provides depth understand ing internetwork ing techniques current internet students study vari ous routing switching algorithms protocols including tra inter routing router switc h architecture switch scheduling traffic engineering students also learn hands operation typical routers switches topics introduction routing algorithms network flow optimization routing protocols ip address lookup packet classification switch architecture packet queuing scheduling traffic conditioning textbook deepankar medhi karthikeyan ramasamy network routing algorithms protocols architectures morgan kaufmann h jonathan chao bin liu high perfor mance switches routers wiley ieee press last update deng pan</t>
+          <t>tcn mobile wireless networks catalog description techniques design operation wireless networks lans mans wans analytical models application traffic mobility models mobility control wireless atm credits prerequisites tcn equivalent type elective mstn mscs ms ph students course objectives course provides students fundame ntal knowledge key techniques design operation mobile wireless networks focusing upper layers various wireless networks course cove rs analytical models routing algorithms scheduling algorithms mac protocols congestion control algorithms cross layer design qos provisioning well selected pics cutting edge wireless networking research topics transmission fundamentals communication networks satellite communications cellular networks mobile ip wap wlans introduction phy cross layer design introduction optimization pplication comm unication networks selected topics wireless networking research textbook william stallings wireless communication networks nd edition prentice hall last update shaolei ren</t>
         </is>
       </c>
     </row>
     <row r="207">
       <c r="A207" t="inlineStr">
         <is>
-          <t>TCN_6270</t>
+          <t>TCN_6275</t>
         </is>
       </c>
       <c r="B207" t="inlineStr">
         <is>
-          <t>tcn mobile wireless networks catalog description techniques design operation wireless networks lans mans wans analytical models application traffic mobility models mobility control wireless atm credits prerequisites tcn equivalent type elective mstn mscs ms ph students course objectives course provides students fundame ntal knowledge key techniques design operation mobile wireless networks focusing upper layers various wireless networks course cove rs analytical models routing algorithms scheduling algorithms mac protocols congestion control algorithms cross layer design qos provisioning well selected pics cutting edge wireless networking research topics transmission fundamentals communication networks satellite communications cellular networks mobile ip wap wlans introduction phy cross layer design introduction optimization pplication comm unication networks selected topics wireless networking research textbook william stallings wireless communication networks nd edition prentice hall last update shaolei ren</t>
+          <t>tcn mobile computing catalog description enabling technologies impediments mobile computing credits prerequisites graduate standing permission instructor type required mstn course objectives course explores enabling technologies impediments mobile computing cellular systems described multiple generations g g g including emerging fifth generation providing range mobility management solutions impediments mobile environment covered course also explores research issues pervasive computing close relative ubiquitous computing examines young rich body exciting ideas solutions paradigm shifts many traditional areas telecommunications networking computer science engineering information technology others impacted constraints demands mobile pervasive computing includi ng limited energy management hence problems limitations due impediments explained review recent literature cate gories identify problems attempt solve course understand th e literature define new problems provide solutions finally provide evaluation th e solutions objective course threefold expose important prior results field illustrate current trends advancements future direction give practical ex perience area design execution modest research project topics include mobile networking personal communication systems smart devices mobile applications topics introduction research road map constraints demands mobile computing emerging mobile computing paradigms personal communication systems generation cellular systems gsm mobility management location tracking systems evolution g g systems umts lte g cellular systems wireless networks location management ad hoc networks security issues mobile ad hoc networks pervasive ubiquitous computing case studies emerging standards textbook course textbook instead cover number original research papers important read digest paper th e class website contains links references material help student digest material presented class last update dr niki pissinou</t>
         </is>
       </c>
     </row>
     <row r="208">
       <c r="A208" t="inlineStr">
         <is>
-          <t>TCN_6275</t>
+          <t>TCN_6420</t>
         </is>
       </c>
       <c r="B208" t="inlineStr">
         <is>
-          <t>tcn mobile computing catalog description enabling technologies impediments mobile computing credits prerequisites graduate standing permission instructor type required mstn course objectives course explores enabling technologies impediments mobile computing cellular systems described multiple generations g g g including emerging fifth generation providing range mobility management solutions impediments mobile environment covered course also explores research issues pervasive computing close relative ubiquitous computing examines young rich body exciting ideas solutions paradigm shifts many traditional areas telecommunications networking computer science engineering information technology others impacted constraints demands mobile pervasive computing includi ng limited energy management hence problems limitations due impediments explained review recent literature cate gories identify problems attempt solve course understand th e literature define new problems provide solutions finally provide evaluation th e solutions objective course threefold expose important prior results field illustrate current trends advancements future direction give practical ex perience area design execution modest research project topics include mobile networking personal communication systems smart devices mobile applications topics introduction research road map constraints demands mobile computing emerging mobile computing paradigms personal communication systems generation cellular systems gsm mobility management location tracking systems evolution g g systems umts lte g cellular systems wireless networks location management ad hoc networks security issues mobile ad hoc networks pervasive ubiquitous computing case studies emerging standards textbook course textbook instead cover number original research papers important read digest paper th e class website contains links references material help student digest material presented class last update dr niki pissinou</t>
+          <t>tcn modeling perf ormance evaluation telecommunication networks catalog description course covers methods research issues models performance evaluation high speed cellular netw orks focuses tools markov queues queuing networks theory applications credits prerequisites tcn computer communications ne tworking technologies equivalent type elective msit mstn mscs course objectives students learn techniques reasoning nd analyzing performance computer communication network systems includi ng mathematical models e g probability statistics queuing theory simulation topics introduction performance evaluation measurement techniques tools probability statistics simulation queuing models experimental design analysis topics prac tical subject matters textbook discrete event system simulation jerry banks john carson ii barry nelson david nicol prentice hall june isbn last update jason liu</t>
         </is>
       </c>
     </row>
     <row r="209">
       <c r="A209" t="inlineStr">
         <is>
-          <t>TCN_6420</t>
+          <t>TCN_6430</t>
         </is>
       </c>
       <c r="B209" t="inlineStr">
         <is>
-          <t>tcn modeling perf ormance evaluation telecommunication networks catalog description course covers methods research issues models performance evaluation high speed cellular netw orks focuses tools markov queues queuing networks theory applications credits prerequisites tcn computer communications ne tworking technologies equivalent type elective msit mstn mscs course objectives students learn techniques reasoning nd analyzing performance computer communication network systems includi ng mathematical models e g probability statistics queuing theory simulation topics introduction performance evaluation measurement techniques tools probability statistics simulation queuing models experimental design analysis topics prac tical subject matters textbook discrete event system simulation jerry banks john carson ii barry nelson david nicol prentice hall june isbn last update jason liu</t>
+          <t>tcn networks manageme nt control standards catalog description protocols management telecom netw orks including simple network management protocol common management informati protocol extensio n protocols optimize network performance credits prerequisites tcn equivalent type required mstn system administration track course msit course objectives course provides students compre hensive view network management problem including concepts challenges dime nsions models techniques covers network management technologies e g snmp widely used today also introduces students emerging technol ogies e g openflow research field topics review important network elements scope challenges network management iso telecommunications management netw ork model framework network management fcaps simple network management protocol snmp software defined networking openflow textbook required none recommended douglas comer automated network management systems prentice hall alexander clemm network management fundamentals cisco press last update xin sun</t>
         </is>
       </c>
     </row>
     <row r="210">
       <c r="A210" t="inlineStr">
         <is>
-          <t>TCN_6430</t>
+          <t>TCN_6450</t>
         </is>
       </c>
       <c r="B210" t="inlineStr">
         <is>
-          <t>tcn networks manageme nt control standards catalog description protocols management telecom netw orks including simple network management protocol common management informati protocol extensio n protocols optimize network performance credits prerequisites tcn equivalent type required mstn system administration track course msit course objectives course provides students compre hensive view network management problem including concepts challenges dime nsions models techniques covers network management technologies e g snmp widely used today also introduces students emerging technol ogies e g openflow research field topics review important network elements scope challenges network management iso telecommunications management netw ork model framework network management fcaps simple network management protocol snmp software defined networking openflow textbook required none recommended douglas comer automated network management systems prentice hall alexander clemm network management fundamentals cisco press last update xin sun</t>
+          <t>tcn wireless information systems catalog description enabling technologies impediments wi reless information systems focuses software architectures information nd location management wireless environment credits prerequisites graduate standing permission instructor type elective mstn course objectives enabling technologies impediments wire less pervasive ubiqui tous wearable information systems impediments wis environment covered set explore young rich body exciting ideas solutions paradigm shifts problems limitations due impe diments explained students review recent literature categories identify problems attempt solve approach understand area sociated literature define new problems provide solutions fi nally provide evaluation solutions topics introduction wis models wis architectural design service oriented context oriented safety oriented wis models service discovery models broadcasting air indexing mobile databases wireless data caching moving objects trajectory privacy trajectory sensor objects wearable wireless sensing systems wis security privacy adaptive mobile applications mobile software development models peer peer systems case studies emerging standards textbook course textbook instead cover number original research papers important students read digest paper class website contains links references material help student digest material presented class last update dr niki pissinou</t>
         </is>
       </c>
     </row>
     <row r="211">
       <c r="A211" t="inlineStr">
         <is>
-          <t>TCN_6450</t>
+          <t>TCN_6880</t>
         </is>
       </c>
       <c r="B211" t="inlineStr">
-        <is>
-          <t>tcn wireless information systems catalog description enabling technologies impediments wi reless information systems focuses software architectures information nd location management wireless environment credits prerequisites graduate standing permission instructor type elective mstn course objectives enabling technologies impediments wire less pervasive ubiqui tous wearable information systems impediments wis environment covered set explore young rich body exciting ideas solutions paradigm shifts problems limitations due impe diments explained students review recent literature categories identify problems attempt solve approach understand area sociated literature define new problems provide solutions fi nally provide evaluation solutions topics introduction wis models wis architectural design service oriented context oriented safety oriented wis models service discovery models broadcasting air indexing mobile databases wireless data caching moving objects trajectory privacy trajectory sensor objects wearable wireless sensing systems wis security privacy adaptive mobile applications mobile software development models peer peer systems case studies emerging standards textbook course textbook instead cover number original research papers important students read digest paper class website contains links references material help student digest material presented class last update dr niki pissinou</t>
-        </is>
-      </c>
-    </row>
-    <row r="212">
-      <c r="A212" t="inlineStr">
-        <is>
-          <t>TCN_6880</t>
-        </is>
-      </c>
-      <c r="B212" t="inlineStr">
         <is>
           <t>tcn telecommunications public policy development standards catalog description concept oriented examination dom estic international telecommunications policy processes standards setting environment credits prerequisites graduate standing permission instructor type elective mstn course objectives course covers public policy issues lated telecomm unications networking information technology industries including internet historical present future perspective addresses e volution telecom industry public policy impact reshaping world nd importance government regulations management technical decisions th ese industries examples include privacy electronic signatures digital divide bandwid th auctions ip telephone internet taxation wireless communication students lear n legal regulatory history industry better understand current ssues confronting marketplace lectures discussions project analyses students gain basic understanding telecommunications public policy bei ng developed well current issues topics history development telecommunicati ons industry firms regulated natural monopoly market power economies scale scope public interest concepts regulatory capture regulation vs antitrust network externalities overview services play ers access services toll local regulated regulates traditiona l rate return regulation revenue requirement value service pricing tr aditional patterns cross subsidy early history telecommunications co mmunications act partial history consent decree slow development competition divestiture divestiture access changes alternative regulatory frameworks telecom act fcc orders economics networks regulations economics scale scope sunk costs barriers entry unbundled network elements regulation deregulation teleco act effect government regulation framework competition competition local services facilitie based competition regulation based competition wireline wireless competition residential local long distance bundling residential local long distance competition mobile wireless comm unications competition wireless winning strategies mobile handset market value chain internet commerce wireless world competition service look creasingly like commodity little differentiation auction theory spectrum truly scarce auctioning spectrum benefit consumers global competition internationa l regulations act effect convergence telecom comp anies computer hardware software companies cable operators compete voice da ta traffic integration networks emerging issues privacy security privacy etc textbook jame harry green irwin handbook telecommunications th edition mcgraw hill professional international telecommunication regulations itu instructor post readings website readings posted instructor notify student supplementary material assi gned class nearly world wide web cla ss website students responsible using uniform resource location url addresses provided website locate assigned material course syllabus web links assi gned reading material last update dr niki pissinou</t>
         </is>

</xml_diff>